<commit_message>
bd : instantane apres verification de production
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-08-20 11:10</t>
+    <t>2026-08-20 11:19</t>
   </si>
   <si>
     <t>Squads</t>
@@ -134,7 +134,7 @@
     <t>non</t>
   </si>
   <si>
-    <t>2026-08-20 11:04</t>
+    <t>2026-08-20 11:18</t>
   </si>
   <si>
     <t>MBENG Ivan</t>

</xml_diff>

<commit_message>
Cycle de livraison, bande passante, rallonges et statistiques
- workflow metier : faisabilite, implementation, test qualif, retour qualif,
  test business, retour business, DAB, CAB ACL, CAB GO LIVE, live, incident
- chaque changement de statut est historise avec son auteur
- histogramme horizontal de bande passante par porteur (consomme, engage,
  marge libre) base sur la capacite calendaire et les rallonges
- demande de rallonge par le developpeur, decision du Scrum Master : les heures
  accordees s ajoutent au point, avec report possible sur une autre semaine
- espace Mes realisations : statistiques par sprint et globales, synthese
  test business / en cours / deploiement / go live / corrections / incidents
- 109 tests fonctionnels

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="140">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-08-20 11:19</t>
+    <t>2026-08-20 17:04</t>
   </si>
   <si>
     <t>Squads</t>
@@ -68,13 +68,13 @@
     <t>Créée le</t>
   </si>
   <si>
-    <t>Squad CX Kaabu</t>
+    <t>Squad Digital</t>
   </si>
   <si>
     <t>2026-08-20</t>
   </si>
   <si>
-    <t>Squad Digital</t>
+    <t>Squad Test 1787245020398</t>
   </si>
   <si>
     <t>Nom</t>
@@ -134,7 +134,7 @@
     <t>non</t>
   </si>
   <si>
-    <t>2026-08-20 11:18</t>
+    <t>2026-08-20 16:56</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -266,10 +266,10 @@
     <t>Passage en déploiement preprod + test des requêtes</t>
   </si>
   <si>
-    <t>En cours</t>
-  </si>
-  <si>
-    <t>2026-08-20 09:07</t>
+    <t>IMPLEMENTATION</t>
+  </si>
+  <si>
+    <t>2026-08-20 16:47</t>
   </si>
   <si>
     <t>#9322</t>
@@ -281,9 +281,6 @@
     <t>Livraison de la fonctionnalité d'import</t>
   </si>
   <si>
-    <t>2026-08-20 08:36</t>
-  </si>
-  <si>
     <t>Appui — recouvrement LOT 1</t>
   </si>
   <si>
@@ -293,7 +290,7 @@
     <t>Bloqué / hors capacité</t>
   </si>
   <si>
-    <t>2026-08-20 10:47</t>
+    <t>2026-08-20 11:46</t>
   </si>
   <si>
     <t>#11419</t>
@@ -312,6 +309,9 @@
   </si>
   <si>
     <t>Supervision technique + revue des livraisons</t>
+  </si>
+  <si>
+    <t>Non démarré</t>
   </si>
   <si>
     <t>Date</t>
@@ -906,7 +906,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -965,10 +965,10 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -982,10 +982,10 @@
         <v>8</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
@@ -1046,7 +1046,7 @@
         <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
         <v>28</v>
@@ -1069,7 +1069,7 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E3" t="s">
         <v>28</v>
@@ -1092,7 +1092,7 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
         <v>28</v>
@@ -1115,7 +1115,7 @@
         <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
         <v>28</v>
@@ -1138,7 +1138,7 @@
         <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E6" t="s">
         <v>28</v>
@@ -1161,7 +1161,7 @@
         <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E7" t="s">
         <v>28</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>53</v>
@@ -1283,7 +1283,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>53</v>
@@ -1309,7 +1309,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>53</v>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
         <v>53</v>
@@ -1435,7 +1435,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>53</v>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>53</v>
@@ -1524,12 +1524,12 @@
         <v>29</v>
       </c>
       <c r="O3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
         <v>53</v>
@@ -1547,36 +1547,36 @@
         <v>29</v>
       </c>
       <c r="G4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" t="s">
         <v>88</v>
-      </c>
-      <c r="H4" t="s">
-        <v>89</v>
       </c>
       <c r="I4">
         <v>160</v>
       </c>
-      <c r="J4">
-        <v>45</v>
+      <c r="J4" t="s">
+        <v>29</v>
       </c>
       <c r="K4" t="s">
+        <v>89</v>
+      </c>
+      <c r="L4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" t="s">
         <v>90</v>
-      </c>
-      <c r="L4" t="s">
-        <v>28</v>
-      </c>
-      <c r="M4" t="s">
-        <v>29</v>
-      </c>
-      <c r="N4" t="s">
-        <v>29</v>
-      </c>
-      <c r="O4" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
         <v>53</v>
@@ -1588,16 +1588,16 @@
         <v>39</v>
       </c>
       <c r="E5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" t="s">
         <v>92</v>
       </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>93</v>
-      </c>
-      <c r="H5" t="s">
-        <v>94</v>
       </c>
       <c r="I5">
         <v>84</v>
@@ -1623,7 +1623,7 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
         <v>53</v>
@@ -1635,16 +1635,16 @@
         <v>30</v>
       </c>
       <c r="E6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" t="s">
         <v>95</v>
       </c>
-      <c r="F6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>96</v>
-      </c>
-      <c r="H6" t="s">
-        <v>97</v>
       </c>
       <c r="I6">
         <v>60</v>
@@ -1653,7 +1653,7 @@
         <v>29</v>
       </c>
       <c r="K6" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="L6" t="s">
         <v>37</v>
@@ -1665,7 +1665,7 @@
         <v>29</v>
       </c>
       <c r="O6" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bd : instantane apres mise en service du cycle de livraison
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="139">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-08-20 17:04</t>
+    <t>2026-08-20 17:09</t>
   </si>
   <si>
     <t>Squads</t>
@@ -74,9 +74,6 @@
     <t>2026-08-20</t>
   </si>
   <si>
-    <t>Squad Test 1787245020398</t>
-  </si>
-  <si>
     <t>Nom</t>
   </si>
   <si>
@@ -134,7 +131,7 @@
     <t>non</t>
   </si>
   <si>
-    <t>2026-08-20 16:56</t>
+    <t>2026-08-20 17:07</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -858,7 +855,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -933,7 +930,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -971,23 +968,6 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3">
-        <v>8</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1014,163 +994,163 @@
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>21</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
       </c>
       <c r="D2" t="s">
         <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
         <v>30</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>31</v>
-      </c>
-      <c r="C3" t="s">
-        <v>32</v>
       </c>
       <c r="D3" t="s">
         <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
         <v>34</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>35</v>
-      </c>
-      <c r="C4" t="s">
-        <v>36</v>
       </c>
       <c r="D4" t="s">
         <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" t="s">
         <v>37</v>
-      </c>
-      <c r="G4" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" t="s">
         <v>39</v>
       </c>
-      <c r="B5" t="s">
-        <v>40</v>
-      </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
         <v>41</v>
       </c>
-      <c r="B6" t="s">
-        <v>42</v>
-      </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
         <v>44</v>
       </c>
-      <c r="B7" t="s">
-        <v>45</v>
-      </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1195,22 +1175,22 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1218,13 +1198,13 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
         <v>53</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>54</v>
-      </c>
-      <c r="D2" t="s">
-        <v>55</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -1233,7 +1213,7 @@
         <v>600</v>
       </c>
       <c r="G2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1260,25 +1240,25 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1286,16 +1266,16 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" t="s">
         <v>53</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>60</v>
-      </c>
-      <c r="D2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E2" t="s">
-        <v>61</v>
       </c>
       <c r="F2">
         <v>5</v>
@@ -1304,7 +1284,7 @@
         <v>200</v>
       </c>
       <c r="H2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1312,16 +1292,16 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" t="s">
         <v>62</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>63</v>
-      </c>
-      <c r="E3" t="s">
-        <v>64</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -1330,7 +1310,7 @@
         <v>200</v>
       </c>
       <c r="H3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1338,16 +1318,16 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" t="s">
         <v>65</v>
       </c>
-      <c r="D4" t="s">
-        <v>66</v>
-      </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F4">
         <v>5</v>
@@ -1356,7 +1336,7 @@
         <v>200</v>
       </c>
       <c r="H4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1391,46 +1371,46 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1438,46 +1418,46 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
         <v>79</v>
       </c>
-      <c r="F2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>80</v>
-      </c>
-      <c r="H2" t="s">
-        <v>81</v>
       </c>
       <c r="I2">
         <v>35</v>
       </c>
       <c r="J2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" t="s">
         <v>82</v>
-      </c>
-      <c r="L2" t="s">
-        <v>37</v>
-      </c>
-      <c r="M2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1485,46 +1465,46 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" t="s">
         <v>84</v>
       </c>
-      <c r="F3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>85</v>
-      </c>
-      <c r="H3" t="s">
-        <v>86</v>
       </c>
       <c r="I3">
         <v>160</v>
       </c>
       <c r="J3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K3" t="s">
+        <v>81</v>
+      </c>
+      <c r="L3" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3" t="s">
         <v>82</v>
-      </c>
-      <c r="L3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N3" t="s">
-        <v>29</v>
-      </c>
-      <c r="O3" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1532,46 +1512,46 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G4" t="s">
+        <v>86</v>
+      </c>
+      <c r="H4" t="s">
         <v>87</v>
-      </c>
-      <c r="H4" t="s">
-        <v>88</v>
       </c>
       <c r="I4">
         <v>160</v>
       </c>
       <c r="J4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K4" t="s">
+        <v>88</v>
+      </c>
+      <c r="L4" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O4" t="s">
         <v>89</v>
-      </c>
-      <c r="L4" t="s">
-        <v>37</v>
-      </c>
-      <c r="M4" t="s">
-        <v>29</v>
-      </c>
-      <c r="N4" t="s">
-        <v>29</v>
-      </c>
-      <c r="O4" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1579,46 +1559,46 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
         <v>91</v>
       </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>92</v>
-      </c>
-      <c r="H5" t="s">
-        <v>93</v>
       </c>
       <c r="I5">
         <v>84</v>
       </c>
       <c r="J5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K5" t="s">
+        <v>81</v>
+      </c>
+      <c r="L5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O5" t="s">
         <v>82</v>
-      </c>
-      <c r="L5" t="s">
-        <v>37</v>
-      </c>
-      <c r="M5" t="s">
-        <v>29</v>
-      </c>
-      <c r="N5" t="s">
-        <v>29</v>
-      </c>
-      <c r="O5" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1626,46 +1606,46 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" t="s">
         <v>94</v>
       </c>
-      <c r="F6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>95</v>
-      </c>
-      <c r="H6" t="s">
-        <v>96</v>
       </c>
       <c r="I6">
         <v>60</v>
       </c>
       <c r="J6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1688,268 +1668,268 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
         <v>102</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>103</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>104</v>
-      </c>
-      <c r="D2" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" t="s">
         <v>106</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" t="s">
         <v>107</v>
-      </c>
-      <c r="C3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D3" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" t="s">
         <v>109</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" t="s">
         <v>110</v>
-      </c>
-      <c r="C4" t="s">
-        <v>104</v>
-      </c>
-      <c r="D4" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" t="s">
         <v>112</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" t="s">
         <v>113</v>
-      </c>
-      <c r="C5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D5" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" t="s">
         <v>115</v>
       </c>
-      <c r="B6" t="s">
-        <v>116</v>
-      </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" t="s">
         <v>117</v>
       </c>
-      <c r="B7" t="s">
-        <v>118</v>
-      </c>
       <c r="C7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" t="s">
         <v>104</v>
-      </c>
-      <c r="D7" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" t="s">
         <v>119</v>
       </c>
-      <c r="B8" t="s">
-        <v>120</v>
-      </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" t="s">
         <v>121</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" t="s">
         <v>122</v>
-      </c>
-      <c r="C9" t="s">
-        <v>104</v>
-      </c>
-      <c r="D9" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B10" t="s">
         <v>124</v>
       </c>
-      <c r="B10" t="s">
-        <v>125</v>
-      </c>
       <c r="C10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" t="s">
         <v>103</v>
       </c>
-      <c r="C11" t="s">
-        <v>104</v>
-      </c>
       <c r="D11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D12" t="s">
         <v>104</v>
-      </c>
-      <c r="D12" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" t="s">
+        <v>103</v>
+      </c>
+      <c r="D13" t="s">
         <v>110</v>
-      </c>
-      <c r="C13" t="s">
-        <v>104</v>
-      </c>
-      <c r="D13" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C14" t="s">
+        <v>103</v>
+      </c>
+      <c r="D14" t="s">
         <v>113</v>
-      </c>
-      <c r="C14" t="s">
-        <v>104</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C16" t="s">
+        <v>103</v>
+      </c>
+      <c r="D16" t="s">
         <v>104</v>
-      </c>
-      <c r="D16" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C17" t="s">
+        <v>103</v>
+      </c>
+      <c r="D17" t="s">
         <v>104</v>
-      </c>
-      <c r="D17" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" t="s">
+        <v>103</v>
+      </c>
+      <c r="D18" t="s">
         <v>133</v>
-      </c>
-      <c r="B18" t="s">
-        <v>122</v>
-      </c>
-      <c r="C18" t="s">
-        <v>104</v>
-      </c>
-      <c r="D18" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B19" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1972,19 +1952,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>138</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Affectation des objectifs par le pilotage
Le super admin et le Scrum Master peuvent creer, modifier, reaffecter, deplacer
d une semaine a l autre et supprimer les objectifs des membres de leur squad.

- droits entree.creer.tous et entree.affecter
- controle de perimetre : porteur actif et rattache a la squad du sprint
- panneau d affectation dans la console, semaine par semaine
- 117 tests fonctionnels

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="142">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-08-20 17:09</t>
+    <t>2026-08-21 10:03</t>
   </si>
   <si>
     <t>Squads</t>
@@ -74,6 +74,12 @@
     <t>2026-08-20</t>
   </si>
   <si>
+    <t>Squad Test 1787306133724</t>
+  </si>
+  <si>
+    <t>2026-08-21</t>
+  </si>
+  <si>
     <t>Nom</t>
   </si>
   <si>
@@ -131,7 +137,7 @@
     <t>non</t>
   </si>
   <si>
-    <t>2026-08-20 17:07</t>
+    <t>2026-08-21 10:00</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -200,9 +206,6 @@
     <t>S1</t>
   </si>
   <si>
-    <t>2026-08-21</t>
-  </si>
-  <si>
     <t>S2</t>
   </si>
   <si>
@@ -278,6 +281,9 @@
     <t>Livraison de la fonctionnalité d'import</t>
   </si>
   <si>
+    <t>2026-08-21 09:07</t>
+  </si>
+  <si>
     <t>Appui — recouvrement LOT 1</t>
   </si>
   <si>
@@ -309,6 +315,9 @@
   </si>
   <si>
     <t>Non démarré</t>
+  </si>
+  <si>
+    <t>2026-08-21 08:10</t>
   </si>
   <si>
     <t>Date</t>
@@ -855,7 +864,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -930,7 +939,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -969,6 +978,23 @@
       </c>
       <c r="E2" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -994,163 +1020,163 @@
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
         <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
         <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
         <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D7" t="s">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1175,22 +1201,22 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1198,13 +1224,13 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -1213,7 +1239,7 @@
         <v>600</v>
       </c>
       <c r="G2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1240,25 +1266,25 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1266,16 +1292,16 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="F2">
         <v>5</v>
@@ -1284,7 +1310,7 @@
         <v>200</v>
       </c>
       <c r="H2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1292,16 +1318,16 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -1310,7 +1336,7 @@
         <v>200</v>
       </c>
       <c r="H3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1318,16 +1344,16 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F4">
         <v>5</v>
@@ -1336,7 +1362,7 @@
         <v>200</v>
       </c>
       <c r="H4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1371,46 +1397,46 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1418,46 +1444,46 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I2">
         <v>35</v>
       </c>
       <c r="J2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1465,46 +1491,46 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I3">
         <v>160</v>
       </c>
-      <c r="J3" t="s">
-        <v>28</v>
+      <c r="J3">
+        <v>20</v>
       </c>
       <c r="K3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1512,46 +1538,46 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I4">
         <v>160</v>
       </c>
       <c r="J4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1559,46 +1585,46 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I5">
         <v>84</v>
       </c>
       <c r="J5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1606,46 +1632,46 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I6">
         <v>60</v>
       </c>
       <c r="J6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="L6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O6" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1668,268 +1694,268 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" t="s">
         <v>106</v>
       </c>
-      <c r="C3" t="s">
-        <v>103</v>
-      </c>
       <c r="D3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B7" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B9" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B10" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D10" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D11" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C12" t="s">
         <v>106</v>
       </c>
-      <c r="C12" t="s">
-        <v>103</v>
-      </c>
       <c r="D12" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C13" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D13" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D14" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B15" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D15" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B16" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D16" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B17" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D17" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B18" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C18" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D18" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B19" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1952,19 +1978,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bd : instantane apres mise en service de l affectation
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="141">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-08-21 10:03</t>
+    <t>2026-08-21 10:08</t>
   </si>
   <si>
     <t>Squads</t>
@@ -74,136 +74,133 @@
     <t>2026-08-20</t>
   </si>
   <si>
-    <t>Squad Test 1787306133724</t>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Rôle</t>
+  </si>
+  <si>
+    <t>Actif</t>
+  </si>
+  <si>
+    <t>Mot de passe à changer</t>
+  </si>
+  <si>
+    <t>Dernière connexion</t>
+  </si>
+  <si>
+    <t>BELINGA Yan</t>
+  </si>
+  <si>
+    <t>yan.belinga@orange.com</t>
+  </si>
+  <si>
+    <t>Développeur</t>
+  </si>
+  <si>
+    <t>oui</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>FOGUE Hervé</t>
+  </si>
+  <si>
+    <t>herve.soubgui@orange.com</t>
+  </si>
+  <si>
+    <t>Tech Lead</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:35</t>
+  </si>
+  <si>
+    <t>FOKA Emmanuel</t>
+  </si>
+  <si>
+    <t>emmanuel.foka@orange.com</t>
+  </si>
+  <si>
+    <t>Super admin</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>2026-08-21 10:06</t>
+  </si>
+  <si>
+    <t>MBENG Ivan</t>
+  </si>
+  <si>
+    <t>ivan.mbeng@orange.com</t>
+  </si>
+  <si>
+    <t>SCHUAME Alexandre</t>
+  </si>
+  <si>
+    <t>alexandre.schuame@orange.com</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:31</t>
+  </si>
+  <si>
+    <t>YAYA Arafat</t>
+  </si>
+  <si>
+    <t>arafat.yaya@orange.com</t>
+  </si>
+  <si>
+    <t>2026-08-20 09:13</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>Début</t>
+  </si>
+  <si>
+    <t>Fin</t>
+  </si>
+  <si>
+    <t>Semaines</t>
+  </si>
+  <si>
+    <t>Capacité (h)</t>
+  </si>
+  <si>
+    <t>Clôturé</t>
+  </si>
+  <si>
+    <t>Sprint #01</t>
+  </si>
+  <si>
+    <t>2026-08-17</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>Semaine</t>
+  </si>
+  <si>
+    <t>Revue</t>
+  </si>
+  <si>
+    <t>Jours ouvrés</t>
+  </si>
+  <si>
+    <t>Clôturée</t>
+  </si>
+  <si>
+    <t>S1</t>
   </si>
   <si>
     <t>2026-08-21</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Rôle</t>
-  </si>
-  <si>
-    <t>Actif</t>
-  </si>
-  <si>
-    <t>Mot de passe à changer</t>
-  </si>
-  <si>
-    <t>Dernière connexion</t>
-  </si>
-  <si>
-    <t>BELINGA Yan</t>
-  </si>
-  <si>
-    <t>yan.belinga@orange.com</t>
-  </si>
-  <si>
-    <t>Développeur</t>
-  </si>
-  <si>
-    <t>oui</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>FOGUE Hervé</t>
-  </si>
-  <si>
-    <t>herve.soubgui@orange.com</t>
-  </si>
-  <si>
-    <t>Tech Lead</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:35</t>
-  </si>
-  <si>
-    <t>FOKA Emmanuel</t>
-  </si>
-  <si>
-    <t>emmanuel.foka@orange.com</t>
-  </si>
-  <si>
-    <t>Super admin</t>
-  </si>
-  <si>
-    <t>non</t>
-  </si>
-  <si>
-    <t>2026-08-21 10:00</t>
-  </si>
-  <si>
-    <t>MBENG Ivan</t>
-  </si>
-  <si>
-    <t>ivan.mbeng@orange.com</t>
-  </si>
-  <si>
-    <t>SCHUAME Alexandre</t>
-  </si>
-  <si>
-    <t>alexandre.schuame@orange.com</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:31</t>
-  </si>
-  <si>
-    <t>YAYA Arafat</t>
-  </si>
-  <si>
-    <t>arafat.yaya@orange.com</t>
-  </si>
-  <si>
-    <t>2026-08-20 09:13</t>
-  </si>
-  <si>
-    <t>Sprint</t>
-  </si>
-  <si>
-    <t>Début</t>
-  </si>
-  <si>
-    <t>Fin</t>
-  </si>
-  <si>
-    <t>Semaines</t>
-  </si>
-  <si>
-    <t>Capacité (h)</t>
-  </si>
-  <si>
-    <t>Clôturé</t>
-  </si>
-  <si>
-    <t>Sprint #01</t>
-  </si>
-  <si>
-    <t>2026-08-17</t>
-  </si>
-  <si>
-    <t>2026-09-04</t>
-  </si>
-  <si>
-    <t>Semaine</t>
-  </si>
-  <si>
-    <t>Revue</t>
-  </si>
-  <si>
-    <t>Jours ouvrés</t>
-  </si>
-  <si>
-    <t>Clôturée</t>
-  </si>
-  <si>
-    <t>S1</t>
   </si>
   <si>
     <t>S2</t>
@@ -864,7 +861,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -939,7 +936,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -978,23 +975,6 @@
       </c>
       <c r="E2" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3">
-        <v>8</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1020,163 +1000,163 @@
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
         <v>26</v>
-      </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>28</v>
       </c>
       <c r="D2" t="s">
         <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
         <v>31</v>
-      </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
-        <v>33</v>
       </c>
       <c r="D3" t="s">
         <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" t="s">
         <v>35</v>
-      </c>
-      <c r="B4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" t="s">
-        <v>37</v>
       </c>
       <c r="D4" t="s">
         <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1201,22 +1181,22 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1224,13 +1204,13 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
         <v>54</v>
-      </c>
-      <c r="C2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" t="s">
-        <v>56</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -1239,7 +1219,7 @@
         <v>600</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1266,25 +1246,25 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1292,16 +1272,16 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="F2">
         <v>5</v>
@@ -1310,7 +1290,7 @@
         <v>200</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1318,16 +1298,16 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" t="s">
         <v>62</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>63</v>
-      </c>
-      <c r="E3" t="s">
-        <v>64</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -1336,7 +1316,7 @@
         <v>200</v>
       </c>
       <c r="H3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1344,16 +1324,16 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" t="s">
         <v>54</v>
-      </c>
-      <c r="C4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" t="s">
-        <v>56</v>
       </c>
       <c r="F4">
         <v>5</v>
@@ -1362,7 +1342,7 @@
         <v>200</v>
       </c>
       <c r="H4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1397,46 +1377,46 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1444,46 +1424,46 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
         <v>79</v>
       </c>
-      <c r="F2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>80</v>
-      </c>
-      <c r="H2" t="s">
-        <v>81</v>
       </c>
       <c r="I2">
         <v>35</v>
       </c>
       <c r="J2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" t="s">
         <v>82</v>
-      </c>
-      <c r="L2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M2" t="s">
-        <v>30</v>
-      </c>
-      <c r="N2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1491,25 +1471,25 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" t="s">
         <v>84</v>
       </c>
-      <c r="F3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>85</v>
-      </c>
-      <c r="H3" t="s">
-        <v>86</v>
       </c>
       <c r="I3">
         <v>160</v>
@@ -1518,19 +1498,19 @@
         <v>20</v>
       </c>
       <c r="K3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="M3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="O3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1538,46 +1518,46 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" t="s">
         <v>88</v>
-      </c>
-      <c r="H4" t="s">
-        <v>89</v>
       </c>
       <c r="I4">
         <v>160</v>
       </c>
       <c r="J4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K4" t="s">
+        <v>89</v>
+      </c>
+      <c r="L4" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O4" t="s">
         <v>90</v>
-      </c>
-      <c r="L4" t="s">
-        <v>38</v>
-      </c>
-      <c r="M4" t="s">
-        <v>30</v>
-      </c>
-      <c r="N4" t="s">
-        <v>30</v>
-      </c>
-      <c r="O4" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1585,46 +1565,46 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
         <v>92</v>
       </c>
-      <c r="F5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>93</v>
-      </c>
-      <c r="H5" t="s">
-        <v>94</v>
       </c>
       <c r="I5">
         <v>84</v>
       </c>
       <c r="J5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K5" t="s">
+        <v>81</v>
+      </c>
+      <c r="L5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O5" t="s">
         <v>82</v>
-      </c>
-      <c r="L5" t="s">
-        <v>38</v>
-      </c>
-      <c r="M5" t="s">
-        <v>30</v>
-      </c>
-      <c r="N5" t="s">
-        <v>30</v>
-      </c>
-      <c r="O5" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1632,46 +1612,46 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" t="s">
         <v>95</v>
       </c>
-      <c r="F6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>96</v>
-      </c>
-      <c r="H6" t="s">
-        <v>97</v>
       </c>
       <c r="I6">
         <v>60</v>
       </c>
       <c r="J6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K6" t="s">
+        <v>97</v>
+      </c>
+      <c r="L6" t="s">
+        <v>36</v>
+      </c>
+      <c r="M6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" t="s">
         <v>98</v>
-      </c>
-      <c r="L6" t="s">
-        <v>38</v>
-      </c>
-      <c r="M6" t="s">
-        <v>30</v>
-      </c>
-      <c r="N6" t="s">
-        <v>30</v>
-      </c>
-      <c r="O6" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1694,268 +1674,268 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>102</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" t="s">
         <v>104</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>105</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>106</v>
-      </c>
-      <c r="D2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" t="s">
         <v>108</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" t="s">
         <v>109</v>
-      </c>
-      <c r="C3" t="s">
-        <v>106</v>
-      </c>
-      <c r="D3" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B4" t="s">
         <v>111</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" t="s">
         <v>112</v>
-      </c>
-      <c r="C4" t="s">
-        <v>106</v>
-      </c>
-      <c r="D4" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" t="s">
         <v>114</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" t="s">
         <v>115</v>
-      </c>
-      <c r="C5" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" t="s">
         <v>117</v>
       </c>
-      <c r="B6" t="s">
-        <v>118</v>
-      </c>
       <c r="C6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" t="s">
         <v>119</v>
       </c>
-      <c r="B7" t="s">
-        <v>120</v>
-      </c>
       <c r="C7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" t="s">
         <v>106</v>
-      </c>
-      <c r="D7" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" t="s">
         <v>121</v>
       </c>
-      <c r="B8" t="s">
-        <v>122</v>
-      </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" t="s">
         <v>123</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D9" t="s">
         <v>124</v>
-      </c>
-      <c r="C9" t="s">
-        <v>106</v>
-      </c>
-      <c r="D9" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" t="s">
         <v>126</v>
       </c>
-      <c r="B10" t="s">
-        <v>127</v>
-      </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" t="s">
         <v>105</v>
       </c>
-      <c r="C11" t="s">
-        <v>106</v>
-      </c>
       <c r="D11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C12" t="s">
+        <v>105</v>
+      </c>
+      <c r="D12" t="s">
         <v>106</v>
-      </c>
-      <c r="D12" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" t="s">
+        <v>105</v>
+      </c>
+      <c r="D13" t="s">
         <v>112</v>
-      </c>
-      <c r="C13" t="s">
-        <v>106</v>
-      </c>
-      <c r="D13" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B14" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" t="s">
         <v>115</v>
-      </c>
-      <c r="C14" t="s">
-        <v>106</v>
-      </c>
-      <c r="D14" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C16" t="s">
+        <v>105</v>
+      </c>
+      <c r="D16" t="s">
         <v>106</v>
-      </c>
-      <c r="D16" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B17" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C17" t="s">
+        <v>105</v>
+      </c>
+      <c r="D17" t="s">
         <v>106</v>
-      </c>
-      <c r="D17" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>134</v>
+      </c>
+      <c r="B18" t="s">
+        <v>123</v>
+      </c>
+      <c r="C18" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" t="s">
         <v>135</v>
-      </c>
-      <c r="B18" t="s">
-        <v>124</v>
-      </c>
-      <c r="C18" t="s">
-        <v>106</v>
-      </c>
-      <c r="D18" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D19" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1978,19 +1958,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>140</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bd : instantane apres ajout du taux de progression
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="139">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-08-21 10:08</t>
+    <t>2026-08-21 15:50</t>
   </si>
   <si>
     <t>Squads</t>
@@ -131,7 +131,7 @@
     <t>non</t>
   </si>
   <si>
-    <t>2026-08-21 10:06</t>
+    <t>2026-08-21 15:48</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -266,7 +266,7 @@
     <t>IMPLEMENTATION</t>
   </si>
   <si>
-    <t>2026-08-20 16:47</t>
+    <t>2026-08-21 11:29</t>
   </si>
   <si>
     <t>#9322</t>
@@ -278,7 +278,7 @@
     <t>Livraison de la fonctionnalité d'import</t>
   </si>
   <si>
-    <t>2026-08-21 09:07</t>
+    <t>2026-08-21 10:46</t>
   </si>
   <si>
     <t>Appui — recouvrement LOT 1</t>
@@ -287,10 +287,7 @@
     <t>Support à la fonctionnalité d'import</t>
   </si>
   <si>
-    <t>Bloqué / hors capacité</t>
-  </si>
-  <si>
-    <t>2026-08-20 11:46</t>
+    <t>2026-08-21 10:54</t>
   </si>
   <si>
     <t>#11419</t>
@@ -302,19 +299,16 @@
     <t>Déploiement preprod + finalisation document DAB</t>
   </si>
   <si>
-    <t>#1322</t>
-  </si>
-  <si>
-    <t>Déploiement du GTR Flow</t>
+    <t>2026-08-21 10:55</t>
+  </si>
+  <si>
+    <t>#0000</t>
   </si>
   <si>
     <t>Supervision technique + revue des livraisons</t>
   </si>
   <si>
-    <t>Non démarré</t>
-  </si>
-  <si>
-    <t>2026-08-21 08:10</t>
+    <t>2026-08-21 10:51</t>
   </si>
   <si>
     <t>Date</t>
@@ -909,7 +903,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1290,7 +1284,7 @@
         <v>200</v>
       </c>
       <c r="H2" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1447,8 +1441,8 @@
       <c r="I2">
         <v>35</v>
       </c>
-      <c r="J2" t="s">
-        <v>28</v>
+      <c r="J2">
+        <v>14</v>
       </c>
       <c r="K2" t="s">
         <v>81</v>
@@ -1541,14 +1535,14 @@
       <c r="I4">
         <v>160</v>
       </c>
-      <c r="J4" t="s">
-        <v>28</v>
+      <c r="J4">
+        <v>34</v>
       </c>
       <c r="K4" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="L4" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="M4" t="s">
         <v>28</v>
@@ -1557,7 +1551,7 @@
         <v>28</v>
       </c>
       <c r="O4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1574,28 +1568,28 @@
         <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F5" t="s">
         <v>28</v>
       </c>
       <c r="G5" t="s">
+        <v>91</v>
+      </c>
+      <c r="H5" t="s">
         <v>92</v>
-      </c>
-      <c r="H5" t="s">
-        <v>93</v>
       </c>
       <c r="I5">
         <v>84</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5">
         <v>28</v>
       </c>
       <c r="K5" t="s">
         <v>81</v>
       </c>
       <c r="L5" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="M5" t="s">
         <v>28</v>
@@ -1604,7 +1598,7 @@
         <v>28</v>
       </c>
       <c r="O5" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1627,22 +1621,22 @@
         <v>28</v>
       </c>
       <c r="G6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" t="s">
         <v>95</v>
-      </c>
-      <c r="H6" t="s">
-        <v>96</v>
       </c>
       <c r="I6">
         <v>60</v>
       </c>
-      <c r="J6" t="s">
-        <v>28</v>
+      <c r="J6">
+        <v>60</v>
       </c>
       <c r="K6" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="L6" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="M6" t="s">
         <v>28</v>
@@ -1651,7 +1645,7 @@
         <v>28</v>
       </c>
       <c r="O6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1674,268 +1668,268 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" t="s">
         <v>103</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>104</v>
-      </c>
-      <c r="C2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D2" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" t="s">
         <v>107</v>
-      </c>
-      <c r="B3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C3" t="s">
-        <v>105</v>
-      </c>
-      <c r="D3" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" t="s">
         <v>110</v>
-      </c>
-      <c r="B4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C4" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" t="s">
         <v>113</v>
-      </c>
-      <c r="B5" t="s">
-        <v>114</v>
-      </c>
-      <c r="C5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D5" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" t="s">
         <v>122</v>
-      </c>
-      <c r="B9" t="s">
-        <v>123</v>
-      </c>
-      <c r="C9" t="s">
-        <v>105</v>
-      </c>
-      <c r="D9" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C11" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D12" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D13" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B14" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B15" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D15" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B16" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C16" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D16" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C17" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B18" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C18" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D18" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B19" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D19" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1958,19 +1952,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>138</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bd : instantane apres reactivation des comptes
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="152">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-08-21 15:50</t>
+    <t>2026-08-22 18:52</t>
   </si>
   <si>
     <t>Squads</t>
@@ -68,6 +68,12 @@
     <t>Créée le</t>
   </si>
   <si>
+    <t>Squad CX Baabu</t>
+  </si>
+  <si>
+    <t>2026-08-22</t>
+  </si>
+  <si>
     <t>Squad Digital</t>
   </si>
   <si>
@@ -131,7 +137,7 @@
     <t>non</t>
   </si>
   <si>
-    <t>2026-08-21 15:48</t>
+    <t>2026-08-22 18:49</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -149,6 +155,18 @@
     <t>2026-08-20 08:31</t>
   </si>
   <si>
+    <t>Sabiatou</t>
+  </si>
+  <si>
+    <t>sabiatou.mfenguie@orange.com</t>
+  </si>
+  <si>
+    <t>Scrum Master</t>
+  </si>
+  <si>
+    <t>2026-08-22 11:48</t>
+  </si>
+  <si>
     <t>YAYA Arafat</t>
   </si>
   <si>
@@ -179,6 +197,12 @@
     <t>Sprint #01</t>
   </si>
   <si>
+    <t>2026-08-24</t>
+  </si>
+  <si>
+    <t>2026-09-11</t>
+  </si>
+  <si>
     <t>2026-08-17</t>
   </si>
   <si>
@@ -200,24 +224,24 @@
     <t>S1</t>
   </si>
   <si>
+    <t>2026-08-28</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>2026-08-31</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>2026-09-07</t>
+  </si>
+  <si>
     <t>2026-08-21</t>
   </si>
   <si>
-    <t>S2</t>
-  </si>
-  <si>
-    <t>2026-08-24</t>
-  </si>
-  <si>
-    <t>2026-08-28</t>
-  </si>
-  <si>
-    <t>S3</t>
-  </si>
-  <si>
-    <t>2026-08-31</t>
-  </si>
-  <si>
     <t>Porteur</t>
   </si>
   <si>
@@ -309,6 +333,21 @@
   </si>
   <si>
     <t>2026-08-21 10:51</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>00000</t>
+  </si>
+  <si>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>Non démarré</t>
+  </si>
+  <si>
+    <t>2026-08-22 11:50</t>
   </si>
   <si>
     <t>Date</t>
@@ -855,7 +894,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -863,7 +902,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -871,7 +910,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -879,7 +918,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -887,7 +926,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -895,7 +934,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -930,7 +969,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -962,13 +1001,30 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3">
+        <v>6</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -980,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -994,163 +1050,186 @@
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
         <v>29</v>
       </c>
-      <c r="B3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>27</v>
-      </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1162,7 +1241,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1175,22 +1254,22 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1198,22 +1277,45 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="E2">
         <v>3</v>
       </c>
       <c r="F2">
+        <v>120</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
         <v>600</v>
       </c>
-      <c r="G2" t="s">
-        <v>36</v>
+      <c r="G3" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1225,7 +1327,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1240,25 +1342,25 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>50</v>
-      </c>
       <c r="H1" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1266,25 +1368,25 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" t="s">
         <v>59</v>
       </c>
-      <c r="D2" t="s">
-        <v>53</v>
-      </c>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="F2">
         <v>5</v>
       </c>
       <c r="G2">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="H2" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1292,25 +1394,25 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
         <v>62</v>
-      </c>
-      <c r="E3" t="s">
-        <v>63</v>
       </c>
       <c r="F3">
         <v>5</v>
       </c>
       <c r="G3">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="H3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1318,25 +1420,103 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F4">
         <v>5</v>
       </c>
       <c r="G4">
+        <v>40</v>
+      </c>
+      <c r="H4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5">
         <v>200</v>
       </c>
-      <c r="H4" t="s">
-        <v>36</v>
+      <c r="H5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>200</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7">
+        <v>200</v>
+      </c>
+      <c r="H7" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1348,7 +1528,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1371,72 +1551,72 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H2" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="I2">
         <v>35</v>
@@ -1445,45 +1625,45 @@
         <v>14</v>
       </c>
       <c r="K2" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="L2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="H3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="I3">
         <v>160</v>
@@ -1492,45 +1672,45 @@
         <v>20</v>
       </c>
       <c r="K3" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="L3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="H4" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="I4">
         <v>160</v>
@@ -1539,45 +1719,45 @@
         <v>34</v>
       </c>
       <c r="K4" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="L4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O4" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G5" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="H5" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="I5">
         <v>84</v>
@@ -1586,45 +1766,45 @@
         <v>28</v>
       </c>
       <c r="K5" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="L5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O5" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H6" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="I6">
         <v>60</v>
@@ -1633,19 +1813,66 @@
         <v>60</v>
       </c>
       <c r="K6" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="L6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O6" t="s">
-        <v>96</v>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G7" t="s">
+        <v>106</v>
+      </c>
+      <c r="H7" t="s">
+        <v>107</v>
+      </c>
+      <c r="I7">
+        <v>45</v>
+      </c>
+      <c r="J7" t="s">
+        <v>30</v>
+      </c>
+      <c r="K7" t="s">
+        <v>108</v>
+      </c>
+      <c r="L7" t="s">
+        <v>38</v>
+      </c>
+      <c r="M7" t="s">
+        <v>30</v>
+      </c>
+      <c r="N7" t="s">
+        <v>30</v>
+      </c>
+      <c r="O7" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1668,268 +1895,268 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="B2" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D2" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D3" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D4" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D5" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="B6" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D6" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C7" t="s">
         <v>116</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>117</v>
-      </c>
-      <c r="C7" t="s">
-        <v>103</v>
-      </c>
-      <c r="D7" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D8" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="B9" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" t="s">
         <v>123</v>
-      </c>
-      <c r="B10" t="s">
-        <v>124</v>
-      </c>
-      <c r="C10" t="s">
-        <v>103</v>
-      </c>
-      <c r="D10" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D11" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D12" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C13" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D13" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D14" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="B15" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D15" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>143</v>
+      </c>
+      <c r="B16" t="s">
         <v>130</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>116</v>
+      </c>
+      <c r="D16" t="s">
         <v>117</v>
-      </c>
-      <c r="C16" t="s">
-        <v>103</v>
-      </c>
-      <c r="D16" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="B17" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D17" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="B18" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="C18" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D18" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="B19" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D19" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1952,19 +2179,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bd : publication manuelle
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="165">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-08-22 18:52</t>
+    <t>2026-08-25 09:31</t>
   </si>
   <si>
     <t>Squads</t>
@@ -68,12 +68,6 @@
     <t>Créée le</t>
   </si>
   <si>
-    <t>Squad CX Baabu</t>
-  </si>
-  <si>
-    <t>2026-08-22</t>
-  </si>
-  <si>
     <t>Squad Digital</t>
   </si>
   <si>
@@ -113,6 +107,36 @@
     <t/>
   </si>
   <si>
+    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
+  </si>
+  <si>
+    <t>charlene.djoungang@orange.com</t>
+  </si>
+  <si>
+    <t>Observateur</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:50</t>
+  </si>
+  <si>
+    <t>Demo User</t>
+  </si>
+  <si>
+    <t>demo@example.com</t>
+  </si>
+  <si>
+    <t>Super admin</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>2026-08-24 14:28</t>
+  </si>
+  <si>
     <t>FOGUE Hervé</t>
   </si>
   <si>
@@ -131,13 +155,7 @@
     <t>emmanuel.foka@orange.com</t>
   </si>
   <si>
-    <t>Super admin</t>
-  </si>
-  <si>
-    <t>non</t>
-  </si>
-  <si>
-    <t>2026-08-22 18:49</t>
+    <t>2026-08-25 07:53</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -167,6 +185,12 @@
     <t>2026-08-22 11:48</t>
   </si>
   <si>
+    <t>Test User</t>
+  </si>
+  <si>
+    <t>test@example.com</t>
+  </si>
+  <si>
     <t>YAYA Arafat</t>
   </si>
   <si>
@@ -197,51 +221,48 @@
     <t>Sprint #01</t>
   </si>
   <si>
+    <t>2026-08-17</t>
+  </si>
+  <si>
+    <t>2026-09-05</t>
+  </si>
+  <si>
+    <t>Semaine</t>
+  </si>
+  <si>
+    <t>Revue</t>
+  </si>
+  <si>
+    <t>Jours ouvrés</t>
+  </si>
+  <si>
+    <t>Clôturée</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>2026-08-21</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
     <t>2026-08-24</t>
   </si>
   <si>
-    <t>2026-09-11</t>
-  </si>
-  <si>
-    <t>2026-08-17</t>
+    <t>2026-08-28</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>2026-08-31</t>
   </si>
   <si>
     <t>2026-09-04</t>
   </si>
   <si>
-    <t>Semaine</t>
-  </si>
-  <si>
-    <t>Revue</t>
-  </si>
-  <si>
-    <t>Jours ouvrés</t>
-  </si>
-  <si>
-    <t>Clôturée</t>
-  </si>
-  <si>
-    <t>S1</t>
-  </si>
-  <si>
-    <t>2026-08-28</t>
-  </si>
-  <si>
-    <t>S2</t>
-  </si>
-  <si>
-    <t>2026-08-31</t>
-  </si>
-  <si>
-    <t>S3</t>
-  </si>
-  <si>
-    <t>2026-09-07</t>
-  </si>
-  <si>
-    <t>2026-08-21</t>
-  </si>
-  <si>
     <t>Porteur</t>
   </si>
   <si>
@@ -278,7 +299,43 @@
     <t>Mis à jour le</t>
   </si>
   <si>
-    <t>#9673</t>
+    <t>9322</t>
+  </si>
+  <si>
+    <t>CxRecov Lot 1</t>
+  </si>
+  <si>
+    <t>Appui — recouvrement LOT 1 | Frontend</t>
+  </si>
+  <si>
+    <t>Implémentation</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:18</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>Supervision technique + revue des livraisons</t>
+  </si>
+  <si>
+    <t>11419</t>
+  </si>
+  <si>
+    <t>Mesure d'engagement des Clients</t>
+  </si>
+  <si>
+    <t>Déploiement preprod + finalisation document DAB</t>
+  </si>
+  <si>
+    <t>Digitalisation de la gestion du recouvrement LOT 1</t>
+  </si>
+  <si>
+    <t>Livraison de la fonctionnalité d'import</t>
+  </si>
+  <si>
+    <t>9673</t>
   </si>
   <si>
     <t>HLR Manager</t>
@@ -287,67 +344,51 @@
     <t>Passage en déploiement preprod + test des requêtes</t>
   </si>
   <si>
-    <t>IMPLEMENTATION</t>
-  </si>
-  <si>
-    <t>2026-08-21 11:29</t>
-  </si>
-  <si>
-    <t>#9322</t>
-  </si>
-  <si>
-    <t>Digitalisation de la gestion du recouvrement LOT 1</t>
-  </si>
-  <si>
-    <t>Livraison de la fonctionnalité d'import</t>
-  </si>
-  <si>
-    <t>2026-08-21 10:46</t>
-  </si>
-  <si>
-    <t>Appui — recouvrement LOT 1</t>
-  </si>
-  <si>
-    <t>Support à la fonctionnalité d'import</t>
-  </si>
-  <si>
-    <t>2026-08-21 10:54</t>
-  </si>
-  <si>
-    <t>#11419</t>
-  </si>
-  <si>
-    <t>Mesure d'engagement des Clients</t>
-  </si>
-  <si>
-    <t>Déploiement preprod + finalisation document DAB</t>
-  </si>
-  <si>
-    <t>2026-08-21 10:55</t>
-  </si>
-  <si>
-    <t>#0000</t>
-  </si>
-  <si>
-    <t>Supervision technique + revue des livraisons</t>
-  </si>
-  <si>
-    <t>2026-08-21 10:51</t>
-  </si>
-  <si>
-    <t>0000</t>
-  </si>
-  <si>
-    <t>00000</t>
-  </si>
-  <si>
-    <t>TEST</t>
-  </si>
-  <si>
-    <t>Non démarré</t>
-  </si>
-  <si>
-    <t>2026-08-22 11:50</t>
+    <t>Bloqué / hors capacité</t>
+  </si>
+  <si>
+    <t>TECH LEAD</t>
+  </si>
+  <si>
+    <t>supervision technique, revue des codes, deploiement compteur des clics, demande DAB CxRECOV</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:24</t>
+  </si>
+  <si>
+    <t>Compteur des clics</t>
+  </si>
+  <si>
+    <t>livrer la première version testable en preprod, deploiement et finaliser le document du DAB</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:27</t>
+  </si>
+  <si>
+    <t>livraison la fonctionnalité consultation, gestion des interactions, les mails et paiement et terminer la fonctionnalité sur l’import</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:28</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:29</t>
+  </si>
+  <si>
+    <t>Passage en déploiement preprod + test desrequêtes</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:38</t>
+  </si>
+  <si>
+    <t>SQUAD DIGITAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAB : CxRecov, HLR Manager, Compteurs des clis
+BD : CxRecov, Compteurs des clis
+Cahier des Tests : CxRecov, HLR Manager, Compteurs des clis</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:31</t>
   </si>
   <si>
     <t>Date</t>
@@ -500,12 +541,17 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7900"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -527,9 +573,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -894,7 +940,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -902,7 +948,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -910,7 +956,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -918,7 +964,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -926,7 +972,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -934,7 +980,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -942,7 +988,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -969,14 +1015,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
@@ -1001,30 +1047,13 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3">
-        <v>8</v>
-      </c>
-      <c r="C3">
-        <v>6</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1036,7 +1065,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1048,188 +1077,257 @@
     <col min="7" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
         <v>27</v>
       </c>
-      <c r="C2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" t="s">
-        <v>29</v>
-      </c>
       <c r="F2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
         <v>31</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" t="s">
         <v>32</v>
       </c>
-      <c r="C3" t="s">
+      <c r="G3" t="s">
         <v>33</v>
-      </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
         <v>35</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>36</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>37</v>
       </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" t="s">
         <v>38</v>
-      </c>
-      <c r="G4" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" t="s">
         <v>40</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>41</v>
       </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
         <v>49</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" t="s">
         <v>50</v>
       </c>
-      <c r="C8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G8" t="s">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>51</v>
+      </c>
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1241,7 +1339,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1249,27 +1347,27 @@
     <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1277,45 +1375,22 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="E2">
         <v>3</v>
       </c>
       <c r="F2">
-        <v>120</v>
+        <v>600</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>600</v>
-      </c>
-      <c r="G3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1327,7 +1402,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1337,30 +1412,30 @@
     <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="H1" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1368,25 +1443,25 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" t="s">
         <v>67</v>
       </c>
-      <c r="D2" t="s">
-        <v>59</v>
-      </c>
       <c r="E2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F2">
         <v>5</v>
       </c>
       <c r="G2">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1394,25 +1469,25 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E3" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="F3">
         <v>5</v>
       </c>
       <c r="G3">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="H3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1420,103 +1495,25 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F4">
         <v>5</v>
       </c>
       <c r="G4">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="H4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C5" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E5" t="s">
-        <v>73</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>200</v>
-      </c>
-      <c r="H5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" t="s">
-        <v>68</v>
-      </c>
-      <c r="F6">
-        <v>5</v>
-      </c>
-      <c r="G6">
-        <v>200</v>
-      </c>
-      <c r="H6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" t="s">
-        <v>70</v>
-      </c>
-      <c r="E7" t="s">
-        <v>62</v>
-      </c>
-      <c r="F7">
-        <v>5</v>
-      </c>
-      <c r="G7">
-        <v>200</v>
-      </c>
-      <c r="H7" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1528,7 +1525,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1546,189 +1543,189 @@
     <col min="15" max="15" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G2" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="H2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="I2">
-        <v>35</v>
+        <v>160</v>
       </c>
       <c r="J2">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="K2" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="L2" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="M2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="O2" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G3" t="s">
-        <v>92</v>
+        <v>41</v>
       </c>
       <c r="H3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="I3">
-        <v>160</v>
+        <v>60</v>
       </c>
       <c r="J3">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="K3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="L3" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="M3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="O3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="H4" t="s">
+        <v>102</v>
+      </c>
+      <c r="I4">
+        <v>84</v>
+      </c>
+      <c r="J4">
+        <v>28</v>
+      </c>
+      <c r="K4" t="s">
         <v>96</v>
       </c>
-      <c r="I4">
-        <v>160</v>
-      </c>
-      <c r="J4">
-        <v>34</v>
-      </c>
-      <c r="K4" t="s">
-        <v>89</v>
-      </c>
       <c r="L4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="M4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="O4" t="s">
         <v>97</v>
@@ -1736,96 +1733,96 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I5">
-        <v>84</v>
+        <v>160</v>
       </c>
       <c r="J5">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="K5" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="L5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="M5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="O5" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="H6" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="I6">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="J6">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="K6" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="L6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="M6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="O6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1833,46 +1830,281 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I7">
+        <v>60</v>
+      </c>
+      <c r="J7" t="s">
+        <v>28</v>
+      </c>
+      <c r="K7" t="s">
+        <v>96</v>
+      </c>
+      <c r="L7" t="s">
+        <v>32</v>
+      </c>
+      <c r="M7" t="s">
+        <v>28</v>
+      </c>
+      <c r="N7" t="s">
+        <v>28</v>
+      </c>
+      <c r="O7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" t="s">
+        <v>112</v>
+      </c>
+      <c r="H8" t="s">
+        <v>113</v>
+      </c>
+      <c r="I8">
+        <v>84</v>
+      </c>
+      <c r="J8" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" t="s">
+        <v>96</v>
+      </c>
+      <c r="L8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M8" t="s">
+        <v>28</v>
+      </c>
+      <c r="N8" t="s">
+        <v>28</v>
+      </c>
+      <c r="O8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E9" t="s">
+        <v>93</v>
+      </c>
+      <c r="F9" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H9" t="s">
+        <v>115</v>
+      </c>
+      <c r="I9">
+        <v>160</v>
+      </c>
+      <c r="J9" t="s">
+        <v>28</v>
+      </c>
+      <c r="K9" t="s">
+        <v>96</v>
+      </c>
+      <c r="L9" t="s">
+        <v>32</v>
+      </c>
+      <c r="M9" t="s">
+        <v>28</v>
+      </c>
+      <c r="N9" t="s">
+        <v>28</v>
+      </c>
+      <c r="O9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" t="s">
+        <v>93</v>
+      </c>
+      <c r="F10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" t="s">
+        <v>103</v>
+      </c>
+      <c r="H10" t="s">
+        <v>115</v>
+      </c>
+      <c r="I10">
+        <v>160</v>
+      </c>
+      <c r="J10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K10" t="s">
+        <v>96</v>
+      </c>
+      <c r="L10" t="s">
+        <v>32</v>
+      </c>
+      <c r="M10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N10" t="s">
+        <v>28</v>
+      </c>
+      <c r="O10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E11" t="s">
         <v>105</v>
       </c>
-      <c r="F7" t="s">
-        <v>105</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="F11" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" t="s">
         <v>106</v>
       </c>
-      <c r="H7" t="s">
-        <v>107</v>
-      </c>
-      <c r="I7">
-        <v>45</v>
-      </c>
-      <c r="J7" t="s">
-        <v>30</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="H11" t="s">
+        <v>118</v>
+      </c>
+      <c r="I11">
+        <v>84</v>
+      </c>
+      <c r="J11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K11" t="s">
         <v>108</v>
       </c>
-      <c r="L7" t="s">
-        <v>38</v>
-      </c>
-      <c r="M7" t="s">
-        <v>30</v>
-      </c>
-      <c r="N7" t="s">
-        <v>30</v>
-      </c>
-      <c r="O7" t="s">
-        <v>109</v>
+      <c r="L11" t="s">
+        <v>32</v>
+      </c>
+      <c r="M11" t="s">
+        <v>28</v>
+      </c>
+      <c r="N11" t="s">
+        <v>28</v>
+      </c>
+      <c r="O11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" t="s">
+        <v>98</v>
+      </c>
+      <c r="F12" t="s">
+        <v>28</v>
+      </c>
+      <c r="G12" t="s">
+        <v>120</v>
+      </c>
+      <c r="H12" t="s">
+        <v>121</v>
+      </c>
+      <c r="I12">
+        <v>60</v>
+      </c>
+      <c r="J12" t="s">
+        <v>28</v>
+      </c>
+      <c r="K12" t="s">
+        <v>96</v>
+      </c>
+      <c r="L12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M12" t="s">
+        <v>28</v>
+      </c>
+      <c r="N12" t="s">
+        <v>28</v>
+      </c>
+      <c r="O12" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1893,270 +2125,270 @@
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="B2" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="C2" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="B3" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="C3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="C4" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D4" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C5" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D5" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="B6" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D6" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" t="s">
         <v>129</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>130</v>
-      </c>
-      <c r="C7" t="s">
-        <v>116</v>
-      </c>
-      <c r="D7" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="B8" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="C8" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D8" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="B9" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="C9" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D9" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B10" t="s">
+        <v>150</v>
+      </c>
+      <c r="C10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D10" t="s">
         <v>136</v>
-      </c>
-      <c r="B10" t="s">
-        <v>137</v>
-      </c>
-      <c r="C10" t="s">
-        <v>116</v>
-      </c>
-      <c r="D10" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="B11" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="C11" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D11" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="B12" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="C12" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D12" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B13" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="C13" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D13" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="B14" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C14" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D14" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="B15" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="C15" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D15" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>156</v>
+      </c>
+      <c r="B16" t="s">
         <v>143</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>129</v>
+      </c>
+      <c r="D16" t="s">
         <v>130</v>
-      </c>
-      <c r="C16" t="s">
-        <v>116</v>
-      </c>
-      <c r="D16" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="B17" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="C17" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D17" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="B18" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="C18" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D18" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="B19" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="C19" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D19" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2177,21 +2409,21 @@
     <col min="5" max="5" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bd : mise à jour d’un objectif
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="165">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,352 +26,352 @@
     <t>Généré le</t>
   </si>
   <si>
+    <t>2026-08-25 12:28</t>
+  </si>
+  <si>
+    <t>Squads</t>
+  </si>
+  <si>
+    <t>Comptes utilisateurs</t>
+  </si>
+  <si>
+    <t>dont actifs</t>
+  </si>
+  <si>
+    <t>Sprints</t>
+  </si>
+  <si>
+    <t>Semaines de revue</t>
+  </si>
+  <si>
+    <t>Objectifs saisis</t>
+  </si>
+  <si>
+    <t>dont validés</t>
+  </si>
+  <si>
+    <t>Jours fériés enregistrés</t>
+  </si>
+  <si>
+    <t>Congés enregistrés</t>
+  </si>
+  <si>
+    <t>Squad</t>
+  </si>
+  <si>
+    <t>Heures / jour</t>
+  </si>
+  <si>
+    <t>Membres</t>
+  </si>
+  <si>
+    <t>Créée le</t>
+  </si>
+  <si>
+    <t>Squad Digital</t>
+  </si>
+  <si>
+    <t>2026-08-20</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Rôle</t>
+  </si>
+  <si>
+    <t>Actif</t>
+  </si>
+  <si>
+    <t>Mot de passe à changer</t>
+  </si>
+  <si>
+    <t>Dernière connexion</t>
+  </si>
+  <si>
+    <t>BELINGA Yan</t>
+  </si>
+  <si>
+    <t>yan.belinga@orange.com</t>
+  </si>
+  <si>
+    <t>Développeur</t>
+  </si>
+  <si>
+    <t>oui</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
+  </si>
+  <si>
+    <t>charlene.djoungang@orange.com</t>
+  </si>
+  <si>
+    <t>Observateur</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:50</t>
+  </si>
+  <si>
+    <t>Demo User</t>
+  </si>
+  <si>
+    <t>demo@example.com</t>
+  </si>
+  <si>
+    <t>Super admin</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>2026-08-24 14:28</t>
+  </si>
+  <si>
+    <t>FOGUE Hervé</t>
+  </si>
+  <si>
+    <t>herve.soubgui@orange.com</t>
+  </si>
+  <si>
+    <t>Tech Lead</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:35</t>
+  </si>
+  <si>
+    <t>FOKA Emmanuel</t>
+  </si>
+  <si>
+    <t>emmanuel.foka@orange.com</t>
+  </si>
+  <si>
+    <t>2026-08-25 07:53</t>
+  </si>
+  <si>
+    <t>MBENG Ivan</t>
+  </si>
+  <si>
+    <t>ivan.mbeng@orange.com</t>
+  </si>
+  <si>
+    <t>SCHUAME Alexandre</t>
+  </si>
+  <si>
+    <t>alexandre.schuame@orange.com</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:31</t>
+  </si>
+  <si>
+    <t>Sabiatou</t>
+  </si>
+  <si>
+    <t>sabiatou.mfenguie@orange.com</t>
+  </si>
+  <si>
+    <t>Scrum Master</t>
+  </si>
+  <si>
+    <t>2026-08-22 11:48</t>
+  </si>
+  <si>
+    <t>Test User</t>
+  </si>
+  <si>
+    <t>test@example.com</t>
+  </si>
+  <si>
+    <t>YAYA Arafat</t>
+  </si>
+  <si>
+    <t>arafat.yaya@orange.com</t>
+  </si>
+  <si>
+    <t>2026-08-20 09:13</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>Début</t>
+  </si>
+  <si>
+    <t>Fin</t>
+  </si>
+  <si>
+    <t>Semaines</t>
+  </si>
+  <si>
+    <t>Capacité (h)</t>
+  </si>
+  <si>
+    <t>Clôturé</t>
+  </si>
+  <si>
+    <t>Sprint #01</t>
+  </si>
+  <si>
+    <t>2026-08-17</t>
+  </si>
+  <si>
+    <t>2026-09-05</t>
+  </si>
+  <si>
+    <t>Semaine</t>
+  </si>
+  <si>
+    <t>Revue</t>
+  </si>
+  <si>
+    <t>Jours ouvrés</t>
+  </si>
+  <si>
+    <t>Clôturée</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>2026-08-21</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>2026-08-24</t>
+  </si>
+  <si>
+    <t>2026-08-28</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>2026-08-31</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>Porteur</t>
+  </si>
+  <si>
+    <t>Ticket</t>
+  </si>
+  <si>
+    <t>ID Perfit</t>
+  </si>
+  <si>
+    <t>Projet</t>
+  </si>
+  <si>
+    <t>Objectif</t>
+  </si>
+  <si>
+    <t>Cap. (h)</t>
+  </si>
+  <si>
+    <t>Réel (h)</t>
+  </si>
+  <si>
+    <t>Exécution</t>
+  </si>
+  <si>
+    <t>Validé</t>
+  </si>
+  <si>
+    <t>Blocage</t>
+  </si>
+  <si>
+    <t>Commentaire</t>
+  </si>
+  <si>
+    <t>Mis à jour le</t>
+  </si>
+  <si>
+    <t>9322</t>
+  </si>
+  <si>
+    <t>CxRecov Lot 1</t>
+  </si>
+  <si>
+    <t>Appui — recouvrement LOT 1 | Frontend</t>
+  </si>
+  <si>
+    <t>Implémentation</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:18</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>Supervision technique + revue des livraisons</t>
+  </si>
+  <si>
+    <t>11419</t>
+  </si>
+  <si>
+    <t>Mesure d'engagement des Clients</t>
+  </si>
+  <si>
+    <t>Déploiement preprod + finalisation document DAB</t>
+  </si>
+  <si>
+    <t>Digitalisation de la gestion du recouvrement LOT 1</t>
+  </si>
+  <si>
+    <t>Livraison de la fonctionnalité d'import</t>
+  </si>
+  <si>
+    <t>9673</t>
+  </si>
+  <si>
+    <t>HLR Manager</t>
+  </si>
+  <si>
+    <t>Passage en déploiement preprod + test des requêtes</t>
+  </si>
+  <si>
+    <t>Bloqué / hors capacité</t>
+  </si>
+  <si>
+    <t>TECH LEAD</t>
+  </si>
+  <si>
+    <t>supervision technique, revue des codes, deploiement compteur des clics, demande DAB CxRECOV</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:24</t>
+  </si>
+  <si>
+    <t>Compteur des clics</t>
+  </si>
+  <si>
+    <t>livrer la première version testable en preprod, deploiement et finaliser le document du DAB</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:27</t>
+  </si>
+  <si>
+    <t>livraison la fonctionnalité consultation, gestion des interactions, les mails et paiement et terminer la fonctionnalité sur l’import</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:28</t>
+  </si>
+  <si>
     <t>2026-08-25 12:16</t>
-  </si>
-  <si>
-    <t>Squads</t>
-  </si>
-  <si>
-    <t>Comptes utilisateurs</t>
-  </si>
-  <si>
-    <t>dont actifs</t>
-  </si>
-  <si>
-    <t>Sprints</t>
-  </si>
-  <si>
-    <t>Semaines de revue</t>
-  </si>
-  <si>
-    <t>Objectifs saisis</t>
-  </si>
-  <si>
-    <t>dont validés</t>
-  </si>
-  <si>
-    <t>Jours fériés enregistrés</t>
-  </si>
-  <si>
-    <t>Congés enregistrés</t>
-  </si>
-  <si>
-    <t>Squad</t>
-  </si>
-  <si>
-    <t>Heures / jour</t>
-  </si>
-  <si>
-    <t>Membres</t>
-  </si>
-  <si>
-    <t>Créée le</t>
-  </si>
-  <si>
-    <t>Squad Digital</t>
-  </si>
-  <si>
-    <t>2026-08-20</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Rôle</t>
-  </si>
-  <si>
-    <t>Actif</t>
-  </si>
-  <si>
-    <t>Mot de passe à changer</t>
-  </si>
-  <si>
-    <t>Dernière connexion</t>
-  </si>
-  <si>
-    <t>BELINGA Yan</t>
-  </si>
-  <si>
-    <t>yan.belinga@orange.com</t>
-  </si>
-  <si>
-    <t>Développeur</t>
-  </si>
-  <si>
-    <t>oui</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
-  </si>
-  <si>
-    <t>charlene.djoungang@orange.com</t>
-  </si>
-  <si>
-    <t>Observateur</t>
-  </si>
-  <si>
-    <t>non</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:50</t>
-  </si>
-  <si>
-    <t>Demo User</t>
-  </si>
-  <si>
-    <t>demo@example.com</t>
-  </si>
-  <si>
-    <t>Super admin</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>2026-08-24 14:28</t>
-  </si>
-  <si>
-    <t>FOGUE Hervé</t>
-  </si>
-  <si>
-    <t>herve.soubgui@orange.com</t>
-  </si>
-  <si>
-    <t>Tech Lead</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:35</t>
-  </si>
-  <si>
-    <t>FOKA Emmanuel</t>
-  </si>
-  <si>
-    <t>emmanuel.foka@orange.com</t>
-  </si>
-  <si>
-    <t>2026-08-25 07:53</t>
-  </si>
-  <si>
-    <t>MBENG Ivan</t>
-  </si>
-  <si>
-    <t>ivan.mbeng@orange.com</t>
-  </si>
-  <si>
-    <t>SCHUAME Alexandre</t>
-  </si>
-  <si>
-    <t>alexandre.schuame@orange.com</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:31</t>
-  </si>
-  <si>
-    <t>Sabiatou</t>
-  </si>
-  <si>
-    <t>sabiatou.mfenguie@orange.com</t>
-  </si>
-  <si>
-    <t>Scrum Master</t>
-  </si>
-  <si>
-    <t>2026-08-22 11:48</t>
-  </si>
-  <si>
-    <t>Test User</t>
-  </si>
-  <si>
-    <t>test@example.com</t>
-  </si>
-  <si>
-    <t>YAYA Arafat</t>
-  </si>
-  <si>
-    <t>arafat.yaya@orange.com</t>
-  </si>
-  <si>
-    <t>2026-08-20 09:13</t>
-  </si>
-  <si>
-    <t>Sprint</t>
-  </si>
-  <si>
-    <t>Début</t>
-  </si>
-  <si>
-    <t>Fin</t>
-  </si>
-  <si>
-    <t>Semaines</t>
-  </si>
-  <si>
-    <t>Capacité (h)</t>
-  </si>
-  <si>
-    <t>Clôturé</t>
-  </si>
-  <si>
-    <t>Sprint #01</t>
-  </si>
-  <si>
-    <t>2026-08-17</t>
-  </si>
-  <si>
-    <t>2026-09-05</t>
-  </si>
-  <si>
-    <t>Semaine</t>
-  </si>
-  <si>
-    <t>Revue</t>
-  </si>
-  <si>
-    <t>Jours ouvrés</t>
-  </si>
-  <si>
-    <t>Clôturée</t>
-  </si>
-  <si>
-    <t>S1</t>
-  </si>
-  <si>
-    <t>2026-08-21</t>
-  </si>
-  <si>
-    <t>S2</t>
-  </si>
-  <si>
-    <t>2026-08-24</t>
-  </si>
-  <si>
-    <t>2026-08-28</t>
-  </si>
-  <si>
-    <t>S3</t>
-  </si>
-  <si>
-    <t>2026-08-31</t>
-  </si>
-  <si>
-    <t>2026-09-04</t>
-  </si>
-  <si>
-    <t>Porteur</t>
-  </si>
-  <si>
-    <t>Ticket</t>
-  </si>
-  <si>
-    <t>ID Perfit</t>
-  </si>
-  <si>
-    <t>Projet</t>
-  </si>
-  <si>
-    <t>Objectif</t>
-  </si>
-  <si>
-    <t>Cap. (h)</t>
-  </si>
-  <si>
-    <t>Réel (h)</t>
-  </si>
-  <si>
-    <t>Exécution</t>
-  </si>
-  <si>
-    <t>Validé</t>
-  </si>
-  <si>
-    <t>Blocage</t>
-  </si>
-  <si>
-    <t>Commentaire</t>
-  </si>
-  <si>
-    <t>Mis à jour le</t>
-  </si>
-  <si>
-    <t>9322</t>
-  </si>
-  <si>
-    <t>CxRecov Lot 1</t>
-  </si>
-  <si>
-    <t>Appui — recouvrement LOT 1 | Frontend</t>
-  </si>
-  <si>
-    <t>Implémentation</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:18</t>
-  </si>
-  <si>
-    <t>0000</t>
-  </si>
-  <si>
-    <t>Supervision technique + revue des livraisons</t>
-  </si>
-  <si>
-    <t>11419</t>
-  </si>
-  <si>
-    <t>Mesure d'engagement des Clients</t>
-  </si>
-  <si>
-    <t>Déploiement preprod + finalisation document DAB</t>
-  </si>
-  <si>
-    <t>Digitalisation de la gestion du recouvrement LOT 1</t>
-  </si>
-  <si>
-    <t>Livraison de la fonctionnalité d'import</t>
-  </si>
-  <si>
-    <t>9673</t>
-  </si>
-  <si>
-    <t>HLR Manager</t>
-  </si>
-  <si>
-    <t>Passage en déploiement preprod + test des requêtes</t>
-  </si>
-  <si>
-    <t>Bloqué / hors capacité</t>
-  </si>
-  <si>
-    <t>TECH LEAD</t>
-  </si>
-  <si>
-    <t>supervision technique, revue des codes, deploiement compteur des clics, demande DAB CxRECOV</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:24</t>
-  </si>
-  <si>
-    <t>Compteur des clics</t>
-  </si>
-  <si>
-    <t>livrer la première version testable en preprod, deploiement et finaliser le document du DAB</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:27</t>
-  </si>
-  <si>
-    <t>livraison la fonctionnalité consultation, gestion des interactions, les mails et paiement et terminer la fonctionnalité sur l’import</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:28</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:29</t>
   </si>
   <si>
     <t>Passage en déploiement preprod + test desrequêtes</t>
@@ -1994,11 +1994,11 @@
       <c r="I10">
         <v>160</v>
       </c>
-      <c r="J10" t="s">
-        <v>28</v>
+      <c r="J10">
+        <v>45</v>
       </c>
       <c r="K10" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="L10" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
bd : modification d’un compte
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="165">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,352 +26,352 @@
     <t>Généré le</t>
   </si>
   <si>
+    <t>2026-08-25 12:47</t>
+  </si>
+  <si>
+    <t>Squads</t>
+  </si>
+  <si>
+    <t>Comptes utilisateurs</t>
+  </si>
+  <si>
+    <t>dont actifs</t>
+  </si>
+  <si>
+    <t>Sprints</t>
+  </si>
+  <si>
+    <t>Semaines de revue</t>
+  </si>
+  <si>
+    <t>Objectifs saisis</t>
+  </si>
+  <si>
+    <t>dont validés</t>
+  </si>
+  <si>
+    <t>Jours fériés enregistrés</t>
+  </si>
+  <si>
+    <t>Congés enregistrés</t>
+  </si>
+  <si>
+    <t>Squad</t>
+  </si>
+  <si>
+    <t>Heures / jour</t>
+  </si>
+  <si>
+    <t>Membres</t>
+  </si>
+  <si>
+    <t>Créée le</t>
+  </si>
+  <si>
+    <t>Squad Digital</t>
+  </si>
+  <si>
+    <t>2026-08-20</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Rôle</t>
+  </si>
+  <si>
+    <t>Actif</t>
+  </si>
+  <si>
+    <t>Mot de passe à changer</t>
+  </si>
+  <si>
+    <t>Dernière connexion</t>
+  </si>
+  <si>
+    <t>BELINGA Yan</t>
+  </si>
+  <si>
+    <t>yan.belinga@orange.com</t>
+  </si>
+  <si>
+    <t>Développeur</t>
+  </si>
+  <si>
+    <t>oui</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
+  </si>
+  <si>
+    <t>charlene.djoungang@orange.com</t>
+  </si>
+  <si>
+    <t>Observateur</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:50</t>
+  </si>
+  <si>
+    <t>Demo User</t>
+  </si>
+  <si>
+    <t>demo@example.com</t>
+  </si>
+  <si>
+    <t>Super admin</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>2026-08-24 14:28</t>
+  </si>
+  <si>
+    <t>FOGUE Hervé</t>
+  </si>
+  <si>
+    <t>herve.soubgui@orange.com</t>
+  </si>
+  <si>
+    <t>Tech Lead</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:35</t>
+  </si>
+  <si>
+    <t>FOKA Emmanuel</t>
+  </si>
+  <si>
+    <t>emmanuel.foka@orange.com</t>
+  </si>
+  <si>
+    <t>2026-08-25 07:53</t>
+  </si>
+  <si>
+    <t>MBENG Ivan</t>
+  </si>
+  <si>
+    <t>ivan.mbeng@orange.com</t>
+  </si>
+  <si>
+    <t>SCHUAME Alexandre</t>
+  </si>
+  <si>
+    <t>alexandre.schuame@orange.com</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:31</t>
+  </si>
+  <si>
+    <t>Sabiatou</t>
+  </si>
+  <si>
+    <t>sabiatou.mfenguie@orange.com</t>
+  </si>
+  <si>
+    <t>Scrum Master</t>
+  </si>
+  <si>
+    <t>2026-08-22 11:48</t>
+  </si>
+  <si>
+    <t>Test User</t>
+  </si>
+  <si>
+    <t>test@example.com</t>
+  </si>
+  <si>
+    <t>YAYA Arafat</t>
+  </si>
+  <si>
+    <t>arafat.yaya@orange.com</t>
+  </si>
+  <si>
+    <t>2026-08-20 09:13</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>Début</t>
+  </si>
+  <si>
+    <t>Fin</t>
+  </si>
+  <si>
+    <t>Semaines</t>
+  </si>
+  <si>
+    <t>Capacité (h)</t>
+  </si>
+  <si>
+    <t>Clôturé</t>
+  </si>
+  <si>
+    <t>Sprint #01</t>
+  </si>
+  <si>
+    <t>2026-08-17</t>
+  </si>
+  <si>
+    <t>2026-09-05</t>
+  </si>
+  <si>
+    <t>Semaine</t>
+  </si>
+  <si>
+    <t>Revue</t>
+  </si>
+  <si>
+    <t>Jours ouvrés</t>
+  </si>
+  <si>
+    <t>Clôturée</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>2026-08-21</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>2026-08-24</t>
+  </si>
+  <si>
+    <t>2026-08-28</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>2026-08-31</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>Porteur</t>
+  </si>
+  <si>
+    <t>Ticket</t>
+  </si>
+  <si>
+    <t>ID Perfit</t>
+  </si>
+  <si>
+    <t>Projet</t>
+  </si>
+  <si>
+    <t>Objectif</t>
+  </si>
+  <si>
+    <t>Cap. (h)</t>
+  </si>
+  <si>
+    <t>Réel (h)</t>
+  </si>
+  <si>
+    <t>Exécution</t>
+  </si>
+  <si>
+    <t>Validé</t>
+  </si>
+  <si>
+    <t>Blocage</t>
+  </si>
+  <si>
+    <t>Commentaire</t>
+  </si>
+  <si>
+    <t>Mis à jour le</t>
+  </si>
+  <si>
+    <t>9322</t>
+  </si>
+  <si>
+    <t>CxRecov Lot 1</t>
+  </si>
+  <si>
+    <t>Appui — recouvrement LOT 1 | Frontend</t>
+  </si>
+  <si>
+    <t>Implémentation</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:18</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>Supervision technique + revue des livraisons</t>
+  </si>
+  <si>
+    <t>11419</t>
+  </si>
+  <si>
+    <t>Mesure d'engagement des Clients</t>
+  </si>
+  <si>
+    <t>Déploiement preprod + finalisation document DAB</t>
+  </si>
+  <si>
+    <t>Digitalisation de la gestion du recouvrement LOT 1</t>
+  </si>
+  <si>
+    <t>Livraison de la fonctionnalité d'import</t>
+  </si>
+  <si>
+    <t>9673</t>
+  </si>
+  <si>
+    <t>HLR Manager</t>
+  </si>
+  <si>
+    <t>Passage en déploiement preprod + test des requêtes</t>
+  </si>
+  <si>
+    <t>Bloqué / hors capacité</t>
+  </si>
+  <si>
+    <t>TECH LEAD</t>
+  </si>
+  <si>
+    <t>supervision technique, revue des codes, deploiement compteur des clics, demande DAB CxRECOV</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:24</t>
+  </si>
+  <si>
+    <t>Compteur des clics</t>
+  </si>
+  <si>
+    <t>livrer la première version testable en preprod, deploiement et finaliser le document du DAB</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:27</t>
+  </si>
+  <si>
+    <t>livraison la fonctionnalité consultation, gestion des interactions, les mails et paiement et terminer la fonctionnalité sur l’import</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:28</t>
+  </si>
+  <si>
     <t>2026-08-25 12:28</t>
-  </si>
-  <si>
-    <t>Squads</t>
-  </si>
-  <si>
-    <t>Comptes utilisateurs</t>
-  </si>
-  <si>
-    <t>dont actifs</t>
-  </si>
-  <si>
-    <t>Sprints</t>
-  </si>
-  <si>
-    <t>Semaines de revue</t>
-  </si>
-  <si>
-    <t>Objectifs saisis</t>
-  </si>
-  <si>
-    <t>dont validés</t>
-  </si>
-  <si>
-    <t>Jours fériés enregistrés</t>
-  </si>
-  <si>
-    <t>Congés enregistrés</t>
-  </si>
-  <si>
-    <t>Squad</t>
-  </si>
-  <si>
-    <t>Heures / jour</t>
-  </si>
-  <si>
-    <t>Membres</t>
-  </si>
-  <si>
-    <t>Créée le</t>
-  </si>
-  <si>
-    <t>Squad Digital</t>
-  </si>
-  <si>
-    <t>2026-08-20</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Rôle</t>
-  </si>
-  <si>
-    <t>Actif</t>
-  </si>
-  <si>
-    <t>Mot de passe à changer</t>
-  </si>
-  <si>
-    <t>Dernière connexion</t>
-  </si>
-  <si>
-    <t>BELINGA Yan</t>
-  </si>
-  <si>
-    <t>yan.belinga@orange.com</t>
-  </si>
-  <si>
-    <t>Développeur</t>
-  </si>
-  <si>
-    <t>oui</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
-  </si>
-  <si>
-    <t>charlene.djoungang@orange.com</t>
-  </si>
-  <si>
-    <t>Observateur</t>
-  </si>
-  <si>
-    <t>non</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:50</t>
-  </si>
-  <si>
-    <t>Demo User</t>
-  </si>
-  <si>
-    <t>demo@example.com</t>
-  </si>
-  <si>
-    <t>Super admin</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>2026-08-24 14:28</t>
-  </si>
-  <si>
-    <t>FOGUE Hervé</t>
-  </si>
-  <si>
-    <t>herve.soubgui@orange.com</t>
-  </si>
-  <si>
-    <t>Tech Lead</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:35</t>
-  </si>
-  <si>
-    <t>FOKA Emmanuel</t>
-  </si>
-  <si>
-    <t>emmanuel.foka@orange.com</t>
-  </si>
-  <si>
-    <t>2026-08-25 07:53</t>
-  </si>
-  <si>
-    <t>MBENG Ivan</t>
-  </si>
-  <si>
-    <t>ivan.mbeng@orange.com</t>
-  </si>
-  <si>
-    <t>SCHUAME Alexandre</t>
-  </si>
-  <si>
-    <t>alexandre.schuame@orange.com</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:31</t>
-  </si>
-  <si>
-    <t>Sabiatou</t>
-  </si>
-  <si>
-    <t>sabiatou.mfenguie@orange.com</t>
-  </si>
-  <si>
-    <t>Scrum Master</t>
-  </si>
-  <si>
-    <t>2026-08-22 11:48</t>
-  </si>
-  <si>
-    <t>Test User</t>
-  </si>
-  <si>
-    <t>test@example.com</t>
-  </si>
-  <si>
-    <t>YAYA Arafat</t>
-  </si>
-  <si>
-    <t>arafat.yaya@orange.com</t>
-  </si>
-  <si>
-    <t>2026-08-20 09:13</t>
-  </si>
-  <si>
-    <t>Sprint</t>
-  </si>
-  <si>
-    <t>Début</t>
-  </si>
-  <si>
-    <t>Fin</t>
-  </si>
-  <si>
-    <t>Semaines</t>
-  </si>
-  <si>
-    <t>Capacité (h)</t>
-  </si>
-  <si>
-    <t>Clôturé</t>
-  </si>
-  <si>
-    <t>Sprint #01</t>
-  </si>
-  <si>
-    <t>2026-08-17</t>
-  </si>
-  <si>
-    <t>2026-09-05</t>
-  </si>
-  <si>
-    <t>Semaine</t>
-  </si>
-  <si>
-    <t>Revue</t>
-  </si>
-  <si>
-    <t>Jours ouvrés</t>
-  </si>
-  <si>
-    <t>Clôturée</t>
-  </si>
-  <si>
-    <t>S1</t>
-  </si>
-  <si>
-    <t>2026-08-21</t>
-  </si>
-  <si>
-    <t>S2</t>
-  </si>
-  <si>
-    <t>2026-08-24</t>
-  </si>
-  <si>
-    <t>2026-08-28</t>
-  </si>
-  <si>
-    <t>S3</t>
-  </si>
-  <si>
-    <t>2026-08-31</t>
-  </si>
-  <si>
-    <t>2026-09-04</t>
-  </si>
-  <si>
-    <t>Porteur</t>
-  </si>
-  <si>
-    <t>Ticket</t>
-  </si>
-  <si>
-    <t>ID Perfit</t>
-  </si>
-  <si>
-    <t>Projet</t>
-  </si>
-  <si>
-    <t>Objectif</t>
-  </si>
-  <si>
-    <t>Cap. (h)</t>
-  </si>
-  <si>
-    <t>Réel (h)</t>
-  </si>
-  <si>
-    <t>Exécution</t>
-  </si>
-  <si>
-    <t>Validé</t>
-  </si>
-  <si>
-    <t>Blocage</t>
-  </si>
-  <si>
-    <t>Commentaire</t>
-  </si>
-  <si>
-    <t>Mis à jour le</t>
-  </si>
-  <si>
-    <t>9322</t>
-  </si>
-  <si>
-    <t>CxRecov Lot 1</t>
-  </si>
-  <si>
-    <t>Appui — recouvrement LOT 1 | Frontend</t>
-  </si>
-  <si>
-    <t>Implémentation</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:18</t>
-  </si>
-  <si>
-    <t>0000</t>
-  </si>
-  <si>
-    <t>Supervision technique + revue des livraisons</t>
-  </si>
-  <si>
-    <t>11419</t>
-  </si>
-  <si>
-    <t>Mesure d'engagement des Clients</t>
-  </si>
-  <si>
-    <t>Déploiement preprod + finalisation document DAB</t>
-  </si>
-  <si>
-    <t>Digitalisation de la gestion du recouvrement LOT 1</t>
-  </si>
-  <si>
-    <t>Livraison de la fonctionnalité d'import</t>
-  </si>
-  <si>
-    <t>9673</t>
-  </si>
-  <si>
-    <t>HLR Manager</t>
-  </si>
-  <si>
-    <t>Passage en déploiement preprod + test des requêtes</t>
-  </si>
-  <si>
-    <t>Bloqué / hors capacité</t>
-  </si>
-  <si>
-    <t>TECH LEAD</t>
-  </si>
-  <si>
-    <t>supervision technique, revue des codes, deploiement compteur des clics, demande DAB CxRECOV</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:24</t>
-  </si>
-  <si>
-    <t>Compteur des clics</t>
-  </si>
-  <si>
-    <t>livrer la première version testable en preprod, deploiement et finaliser le document du DAB</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:27</t>
-  </si>
-  <si>
-    <t>livraison la fonctionnalité consultation, gestion des interactions, les mails et paiement et terminer la fonctionnalité sur l’import</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:28</t>
-  </si>
-  <si>
-    <t>2026-08-25 12:16</t>
   </si>
   <si>
     <t>Passage en déploiement preprod + test desrequêtes</t>
@@ -1994,11 +1994,11 @@
       <c r="I10">
         <v>160</v>
       </c>
-      <c r="J10">
-        <v>45</v>
+      <c r="J10" t="s">
+        <v>28</v>
       </c>
       <c r="K10" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="L10" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
bd : création d’un compte
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -26,133 +26,133 @@
     <t>Généré le</t>
   </si>
   <si>
+    <t>2026-08-25 13:04</t>
+  </si>
+  <si>
+    <t>Squads</t>
+  </si>
+  <si>
+    <t>Comptes utilisateurs</t>
+  </si>
+  <si>
+    <t>dont actifs</t>
+  </si>
+  <si>
+    <t>Sprints</t>
+  </si>
+  <si>
+    <t>Semaines de revue</t>
+  </si>
+  <si>
+    <t>Objectifs saisis</t>
+  </si>
+  <si>
+    <t>dont validés</t>
+  </si>
+  <si>
+    <t>Jours fériés enregistrés</t>
+  </si>
+  <si>
+    <t>Congés enregistrés</t>
+  </si>
+  <si>
+    <t>Squad</t>
+  </si>
+  <si>
+    <t>Heures / jour</t>
+  </si>
+  <si>
+    <t>Membres</t>
+  </si>
+  <si>
+    <t>Créée le</t>
+  </si>
+  <si>
+    <t>Squad Digital</t>
+  </si>
+  <si>
+    <t>2026-08-20</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Rôle</t>
+  </si>
+  <si>
+    <t>Actif</t>
+  </si>
+  <si>
+    <t>Mot de passe à changer</t>
+  </si>
+  <si>
+    <t>Dernière connexion</t>
+  </si>
+  <si>
+    <t>BELINGA Yan</t>
+  </si>
+  <si>
+    <t>yan.belinga@orange.com</t>
+  </si>
+  <si>
+    <t>Développeur</t>
+  </si>
+  <si>
+    <t>oui</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
+  </si>
+  <si>
+    <t>charlene.djoungang@orange.com</t>
+  </si>
+  <si>
+    <t>Observateur</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:50</t>
+  </si>
+  <si>
+    <t>FOGUE Hervé</t>
+  </si>
+  <si>
+    <t>herve.soubgui@orange.com</t>
+  </si>
+  <si>
+    <t>Tech Lead</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:35</t>
+  </si>
+  <si>
+    <t>FOKA</t>
+  </si>
+  <si>
+    <t>emm.foka@gmail.com</t>
+  </si>
+  <si>
+    <t>Scrum Master</t>
+  </si>
+  <si>
+    <t>FOKA Emmanuel</t>
+  </si>
+  <si>
+    <t>emmanuel.foka@orange.com</t>
+  </si>
+  <si>
+    <t>Super admin</t>
+  </si>
+  <si>
     <t>2026-08-25 12:59</t>
-  </si>
-  <si>
-    <t>Squads</t>
-  </si>
-  <si>
-    <t>Comptes utilisateurs</t>
-  </si>
-  <si>
-    <t>dont actifs</t>
-  </si>
-  <si>
-    <t>Sprints</t>
-  </si>
-  <si>
-    <t>Semaines de revue</t>
-  </si>
-  <si>
-    <t>Objectifs saisis</t>
-  </si>
-  <si>
-    <t>dont validés</t>
-  </si>
-  <si>
-    <t>Jours fériés enregistrés</t>
-  </si>
-  <si>
-    <t>Congés enregistrés</t>
-  </si>
-  <si>
-    <t>Squad</t>
-  </si>
-  <si>
-    <t>Heures / jour</t>
-  </si>
-  <si>
-    <t>Membres</t>
-  </si>
-  <si>
-    <t>Créée le</t>
-  </si>
-  <si>
-    <t>Squad Digital</t>
-  </si>
-  <si>
-    <t>2026-08-20</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Rôle</t>
-  </si>
-  <si>
-    <t>Actif</t>
-  </si>
-  <si>
-    <t>Mot de passe à changer</t>
-  </si>
-  <si>
-    <t>Dernière connexion</t>
-  </si>
-  <si>
-    <t>BELINGA Yan</t>
-  </si>
-  <si>
-    <t>yan.belinga@orange.com</t>
-  </si>
-  <si>
-    <t>Développeur</t>
-  </si>
-  <si>
-    <t>oui</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
-  </si>
-  <si>
-    <t>charlene.djoungang@orange.com</t>
-  </si>
-  <si>
-    <t>Observateur</t>
-  </si>
-  <si>
-    <t>non</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:50</t>
-  </si>
-  <si>
-    <t>Emmanuel FOKA</t>
-  </si>
-  <si>
-    <t>emm.foka@gmail.com</t>
-  </si>
-  <si>
-    <t>Scrum Master</t>
-  </si>
-  <si>
-    <t>FOGUE Hervé</t>
-  </si>
-  <si>
-    <t>herve.soubgui@orange.com</t>
-  </si>
-  <si>
-    <t>Tech Lead</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:35</t>
-  </si>
-  <si>
-    <t>FOKA Emmanuel</t>
-  </si>
-  <si>
-    <t>emmanuel.foka@orange.com</t>
-  </si>
-  <si>
-    <t>Super admin</t>
-  </si>
-  <si>
-    <t>2026-08-25 12:49</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -1160,21 +1160,21 @@
         <v>27</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
@@ -1186,7 +1186,7 @@
         <v>27</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>27</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G6" t="s">
         <v>44</v>
@@ -1645,7 +1645,7 @@
         <v>72</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
         <v>97</v>
@@ -1654,7 +1654,7 @@
         <v>28</v>
       </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H3" t="s">
         <v>98</v>
@@ -1833,7 +1833,7 @@
         <v>74</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
         <v>97</v>

</xml_diff>

<commit_message>
bd : modification d’une squad
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="157">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,126 +26,126 @@
     <t>Généré le</t>
   </si>
   <si>
+    <t>2026-08-27 19:10</t>
+  </si>
+  <si>
+    <t>Squads</t>
+  </si>
+  <si>
+    <t>Comptes utilisateurs</t>
+  </si>
+  <si>
+    <t>dont actifs</t>
+  </si>
+  <si>
+    <t>Sprints</t>
+  </si>
+  <si>
+    <t>Semaines de revue</t>
+  </si>
+  <si>
+    <t>Objectifs saisis</t>
+  </si>
+  <si>
+    <t>dont validés</t>
+  </si>
+  <si>
+    <t>Jours fériés enregistrés</t>
+  </si>
+  <si>
+    <t>Congés enregistrés</t>
+  </si>
+  <si>
+    <t>Squad</t>
+  </si>
+  <si>
+    <t>Heures / jour</t>
+  </si>
+  <si>
+    <t>Membres</t>
+  </si>
+  <si>
+    <t>Créée le</t>
+  </si>
+  <si>
+    <t>Squad Digital</t>
+  </si>
+  <si>
+    <t>2026-08-20</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Rôle</t>
+  </si>
+  <si>
+    <t>Actif</t>
+  </si>
+  <si>
+    <t>Mot de passe à changer</t>
+  </si>
+  <si>
+    <t>Dernière connexion</t>
+  </si>
+  <si>
+    <t>BELINGA Yan</t>
+  </si>
+  <si>
+    <t>yan.belinga@orange.com</t>
+  </si>
+  <si>
+    <t>Développeur</t>
+  </si>
+  <si>
+    <t>oui</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>2026-08-25 15:41</t>
+  </si>
+  <si>
+    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
+  </si>
+  <si>
+    <t>charlene.djoungang@orange.com</t>
+  </si>
+  <si>
+    <t>Observateur</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:50</t>
+  </si>
+  <si>
+    <t>FOGUE Hervé</t>
+  </si>
+  <si>
+    <t>herve.soubgui@orange.com</t>
+  </si>
+  <si>
+    <t>Tech Lead</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:35</t>
+  </si>
+  <si>
+    <t>FOKA Emmanuel</t>
+  </si>
+  <si>
+    <t>emmanuel.foka@orange.com</t>
+  </si>
+  <si>
+    <t>Scrum Master</t>
+  </si>
+  <si>
     <t>2026-08-27 03:49</t>
   </si>
   <si>
-    <t>Squads</t>
-  </si>
-  <si>
-    <t>Comptes utilisateurs</t>
-  </si>
-  <si>
-    <t>dont actifs</t>
-  </si>
-  <si>
-    <t>Sprints</t>
-  </si>
-  <si>
-    <t>Semaines de revue</t>
-  </si>
-  <si>
-    <t>Objectifs saisis</t>
-  </si>
-  <si>
-    <t>dont validés</t>
-  </si>
-  <si>
-    <t>Jours fériés enregistrés</t>
-  </si>
-  <si>
-    <t>Congés enregistrés</t>
-  </si>
-  <si>
-    <t>Squad</t>
-  </si>
-  <si>
-    <t>Heures / jour</t>
-  </si>
-  <si>
-    <t>Membres</t>
-  </si>
-  <si>
-    <t>Créée le</t>
-  </si>
-  <si>
-    <t>Squad Digital</t>
-  </si>
-  <si>
-    <t>2026-08-20</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Rôle</t>
-  </si>
-  <si>
-    <t>Actif</t>
-  </si>
-  <si>
-    <t>Mot de passe à changer</t>
-  </si>
-  <si>
-    <t>Dernière connexion</t>
-  </si>
-  <si>
-    <t>BELINGA Yan</t>
-  </si>
-  <si>
-    <t>yan.belinga@orange.com</t>
-  </si>
-  <si>
-    <t>Développeur</t>
-  </si>
-  <si>
-    <t>oui</t>
-  </si>
-  <si>
-    <t>non</t>
-  </si>
-  <si>
-    <t>2026-08-25 15:41</t>
-  </si>
-  <si>
-    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
-  </si>
-  <si>
-    <t>charlene.djoungang@orange.com</t>
-  </si>
-  <si>
-    <t>Observateur</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:50</t>
-  </si>
-  <si>
-    <t>FOGUE Hervé</t>
-  </si>
-  <si>
-    <t>herve.soubgui@orange.com</t>
-  </si>
-  <si>
-    <t>Tech Lead</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:35</t>
-  </si>
-  <si>
-    <t>FOKA Emmanuel</t>
-  </si>
-  <si>
-    <t>emmanuel.foka@orange.com</t>
-  </si>
-  <si>
-    <t>Scrum Master</t>
-  </si>
-  <si>
-    <t>2026-08-25 15:44</t>
-  </si>
-  <si>
     <t>MBENG Ivan</t>
   </si>
   <si>
@@ -176,7 +176,7 @@
     <t>—</t>
   </si>
   <si>
-    <t>2026-08-27 03:46</t>
+    <t>2026-08-27 19:09</t>
   </si>
   <si>
     <t>Test User</t>
@@ -305,16 +305,13 @@
     <t>Implémentation</t>
   </si>
   <si>
-    <t>2026-08-27 03:41</t>
-  </si>
-  <si>
     <t>0000</t>
   </si>
   <si>
     <t>Supervision technique + revue des livraisons</t>
   </si>
   <si>
-    <t>2026-08-25 08:18</t>
+    <t>2026-08-27 03:51</t>
   </si>
   <si>
     <t>11419</t>
@@ -348,9 +345,6 @@
   </si>
   <si>
     <t>supervision technique, revue des codes, deploiement compteur des clics, demande DAB CxRECOV</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:24</t>
   </si>
   <si>
     <t>Compteur des clics</t>
@@ -371,9 +365,6 @@
     <t xml:space="preserve">DAB : CxRecov, HLR Manager, Compteurs des clis
 BD : CxRecov, Compteurs des clis
 Cahier des Tests : CxRecov, HLR Manager, Compteurs des clis</t>
-  </si>
-  <si>
-    <t>2026-08-25 13:48</t>
   </si>
   <si>
     <t>Date</t>
@@ -1171,7 +1162,7 @@
         <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G5" t="s">
         <v>41</v>
@@ -1349,7 +1340,7 @@
         <v>3</v>
       </c>
       <c r="F2">
-        <v>600</v>
+        <v>564</v>
       </c>
       <c r="G2" t="s">
         <v>28</v>
@@ -1420,7 +1411,7 @@
         <v>5</v>
       </c>
       <c r="G2">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="H2" t="s">
         <v>27</v>
@@ -1446,7 +1437,7 @@
         <v>5</v>
       </c>
       <c r="G3">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="H3" t="s">
         <v>28</v>
@@ -1472,7 +1463,7 @@
         <v>5</v>
       </c>
       <c r="G4">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="H4" t="s">
         <v>28</v>
@@ -1568,9 +1559,6 @@
       <c r="E2" t="s">
         <v>91</v>
       </c>
-      <c r="F2" t="s">
-        <v>44</v>
-      </c>
       <c r="G2" t="s">
         <v>92</v>
       </c>
@@ -1578,7 +1566,7 @@
         <v>93</v>
       </c>
       <c r="I2">
-        <v>160</v>
+        <v>40</v>
       </c>
       <c r="J2">
         <v>34</v>
@@ -1596,7 +1584,7 @@
         <v>44</v>
       </c>
       <c r="O2" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1613,22 +1601,19 @@
         <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F3" t="s">
-        <v>44</v>
+        <v>95</v>
       </c>
       <c r="G3" t="s">
         <v>36</v>
       </c>
       <c r="H3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I3">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="J3">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K3" t="s">
         <v>94</v>
@@ -1643,7 +1628,7 @@
         <v>44</v>
       </c>
       <c r="O3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1660,19 +1645,16 @@
         <v>42</v>
       </c>
       <c r="E4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G4" t="s">
         <v>99</v>
       </c>
-      <c r="F4" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>100</v>
       </c>
-      <c r="H4" t="s">
-        <v>101</v>
-      </c>
       <c r="I4">
-        <v>84</v>
+        <v>40</v>
       </c>
       <c r="J4">
         <v>28</v>
@@ -1690,7 +1672,7 @@
         <v>44</v>
       </c>
       <c r="O4" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1709,17 +1691,14 @@
       <c r="E5" t="s">
         <v>91</v>
       </c>
-      <c r="F5" t="s">
-        <v>44</v>
-      </c>
       <c r="G5" t="s">
+        <v>101</v>
+      </c>
+      <c r="H5" t="s">
         <v>102</v>
       </c>
-      <c r="H5" t="s">
-        <v>103</v>
-      </c>
       <c r="I5">
-        <v>160</v>
+        <v>40</v>
       </c>
       <c r="J5">
         <v>20</v>
@@ -1737,7 +1716,7 @@
         <v>44</v>
       </c>
       <c r="O5" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1754,25 +1733,22 @@
         <v>55</v>
       </c>
       <c r="E6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G6" t="s">
         <v>104</v>
       </c>
-      <c r="F6" t="s">
-        <v>44</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>105</v>
       </c>
-      <c r="H6" t="s">
-        <v>106</v>
-      </c>
       <c r="I6">
-        <v>35</v>
+        <v>17.5</v>
       </c>
       <c r="J6">
         <v>14</v>
       </c>
       <c r="K6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L6" t="s">
         <v>27</v>
@@ -1784,7 +1760,7 @@
         <v>44</v>
       </c>
       <c r="O6" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1801,19 +1777,16 @@
         <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>96</v>
-      </c>
-      <c r="F7" t="s">
-        <v>44</v>
+        <v>95</v>
       </c>
       <c r="G7" t="s">
+        <v>107</v>
+      </c>
+      <c r="H7" t="s">
         <v>108</v>
       </c>
-      <c r="H7" t="s">
-        <v>109</v>
-      </c>
       <c r="I7">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="J7" t="s">
         <v>44</v>
@@ -1831,7 +1804,7 @@
         <v>44</v>
       </c>
       <c r="O7" t="s">
-        <v>110</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -1848,19 +1821,16 @@
         <v>42</v>
       </c>
       <c r="E8" t="s">
-        <v>99</v>
-      </c>
-      <c r="F8" t="s">
-        <v>44</v>
+        <v>98</v>
       </c>
       <c r="G8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I8">
-        <v>84</v>
+        <v>40</v>
       </c>
       <c r="J8" t="s">
         <v>44</v>
@@ -1878,7 +1848,7 @@
         <v>44</v>
       </c>
       <c r="O8" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1897,17 +1867,14 @@
       <c r="E9" t="s">
         <v>91</v>
       </c>
-      <c r="F9" t="s">
-        <v>44</v>
-      </c>
       <c r="G9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I9">
-        <v>160</v>
+        <v>40</v>
       </c>
       <c r="J9" t="s">
         <v>44</v>
@@ -1925,7 +1892,7 @@
         <v>44</v>
       </c>
       <c r="O9" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1944,17 +1911,14 @@
       <c r="E10" t="s">
         <v>91</v>
       </c>
-      <c r="F10" t="s">
-        <v>44</v>
-      </c>
       <c r="G10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I10">
-        <v>160</v>
+        <v>40</v>
       </c>
       <c r="J10" t="s">
         <v>44</v>
@@ -1972,7 +1936,7 @@
         <v>44</v>
       </c>
       <c r="O10" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -1989,25 +1953,22 @@
         <v>55</v>
       </c>
       <c r="E11" t="s">
+        <v>103</v>
+      </c>
+      <c r="G11" t="s">
         <v>104</v>
       </c>
-      <c r="F11" t="s">
-        <v>44</v>
-      </c>
-      <c r="G11" t="s">
-        <v>105</v>
-      </c>
       <c r="H11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I11">
-        <v>84</v>
+        <v>17.5</v>
       </c>
       <c r="J11" t="s">
         <v>44</v>
       </c>
       <c r="K11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L11" t="s">
         <v>28</v>
@@ -2019,7 +1980,7 @@
         <v>44</v>
       </c>
       <c r="O11" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -2036,19 +1997,16 @@
         <v>38</v>
       </c>
       <c r="E12" t="s">
-        <v>96</v>
-      </c>
-      <c r="F12" t="s">
-        <v>44</v>
+        <v>95</v>
       </c>
       <c r="G12" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I12">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="J12">
         <v>45</v>
@@ -2066,7 +2024,7 @@
         <v>44</v>
       </c>
       <c r="O12" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2089,268 +2047,268 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" t="s">
         <v>122</v>
-      </c>
-      <c r="B2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C3" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C6" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D6" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B8" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C8" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D8" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D9" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C10" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D10" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B11" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C11" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C12" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D12" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B13" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C13" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D13" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B14" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C14" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D14" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B15" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C15" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D15" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B16" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D16" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B17" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C17" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D17" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B18" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C18" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D18" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B19" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C19" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D19" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -2373,19 +2331,19 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bd : saisie d’un objectif
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -26,124 +26,124 @@
     <t>Généré le</t>
   </si>
   <si>
+    <t>2026-08-31 08:05</t>
+  </si>
+  <si>
+    <t>Squads</t>
+  </si>
+  <si>
+    <t>Comptes utilisateurs</t>
+  </si>
+  <si>
+    <t>dont actifs</t>
+  </si>
+  <si>
+    <t>Sprints</t>
+  </si>
+  <si>
+    <t>Semaines de revue</t>
+  </si>
+  <si>
+    <t>Objectifs saisis</t>
+  </si>
+  <si>
+    <t>dont validés</t>
+  </si>
+  <si>
+    <t>Jours fériés enregistrés</t>
+  </si>
+  <si>
+    <t>Congés enregistrés</t>
+  </si>
+  <si>
+    <t>Squad</t>
+  </si>
+  <si>
+    <t>Heures / jour</t>
+  </si>
+  <si>
+    <t>Membres</t>
+  </si>
+  <si>
+    <t>Créée le</t>
+  </si>
+  <si>
+    <t>Squad Digital</t>
+  </si>
+  <si>
+    <t>2026-08-20</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Rôle</t>
+  </si>
+  <si>
+    <t>Actif</t>
+  </si>
+  <si>
+    <t>Mot de passe à changer</t>
+  </si>
+  <si>
+    <t>Dernière connexion</t>
+  </si>
+  <si>
+    <t>BELINGA Yan</t>
+  </si>
+  <si>
+    <t>yan.belinga@orange.com</t>
+  </si>
+  <si>
+    <t>Développeur</t>
+  </si>
+  <si>
+    <t>oui</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>2026-08-25 15:41</t>
+  </si>
+  <si>
+    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
+  </si>
+  <si>
+    <t>charlene.djoungang@orange.com</t>
+  </si>
+  <si>
+    <t>Observateur</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:50</t>
+  </si>
+  <si>
+    <t>FOGUE Hervé</t>
+  </si>
+  <si>
+    <t>herve.soubgui@orange.com</t>
+  </si>
+  <si>
+    <t>Tech Lead</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:35</t>
+  </si>
+  <si>
+    <t>FOKA Emmanuel</t>
+  </si>
+  <si>
+    <t>emmanuel.foka@orange.com</t>
+  </si>
+  <si>
+    <t>Scrum Master</t>
+  </si>
+  <si>
     <t>2026-08-31 08:01</t>
-  </si>
-  <si>
-    <t>Squads</t>
-  </si>
-  <si>
-    <t>Comptes utilisateurs</t>
-  </si>
-  <si>
-    <t>dont actifs</t>
-  </si>
-  <si>
-    <t>Sprints</t>
-  </si>
-  <si>
-    <t>Semaines de revue</t>
-  </si>
-  <si>
-    <t>Objectifs saisis</t>
-  </si>
-  <si>
-    <t>dont validés</t>
-  </si>
-  <si>
-    <t>Jours fériés enregistrés</t>
-  </si>
-  <si>
-    <t>Congés enregistrés</t>
-  </si>
-  <si>
-    <t>Squad</t>
-  </si>
-  <si>
-    <t>Heures / jour</t>
-  </si>
-  <si>
-    <t>Membres</t>
-  </si>
-  <si>
-    <t>Créée le</t>
-  </si>
-  <si>
-    <t>Squad Digital</t>
-  </si>
-  <si>
-    <t>2026-08-20</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Rôle</t>
-  </si>
-  <si>
-    <t>Actif</t>
-  </si>
-  <si>
-    <t>Mot de passe à changer</t>
-  </si>
-  <si>
-    <t>Dernière connexion</t>
-  </si>
-  <si>
-    <t>BELINGA Yan</t>
-  </si>
-  <si>
-    <t>yan.belinga@orange.com</t>
-  </si>
-  <si>
-    <t>Développeur</t>
-  </si>
-  <si>
-    <t>oui</t>
-  </si>
-  <si>
-    <t>non</t>
-  </si>
-  <si>
-    <t>2026-08-25 15:41</t>
-  </si>
-  <si>
-    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
-  </si>
-  <si>
-    <t>charlene.djoungang@orange.com</t>
-  </si>
-  <si>
-    <t>Observateur</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:50</t>
-  </si>
-  <si>
-    <t>FOGUE Hervé</t>
-  </si>
-  <si>
-    <t>herve.soubgui@orange.com</t>
-  </si>
-  <si>
-    <t>Tech Lead</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:35</t>
-  </si>
-  <si>
-    <t>FOKA Emmanuel</t>
-  </si>
-  <si>
-    <t>emmanuel.foka@orange.com</t>
-  </si>
-  <si>
-    <t>Scrum Master</t>
-  </si>
-  <si>
-    <t>2026-08-28 08:39</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -1291,7 +1291,7 @@
         <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G5" t="s">
         <v>41</v>

</xml_diff>

<commit_message>
bd : création d’un sprint
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="221">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-09-01 11:15</t>
+    <t>2026-09-01 11:29</t>
   </si>
   <si>
     <t>Squads</t>
@@ -74,6 +74,12 @@
     <t>2026-08-20</t>
   </si>
   <si>
+    <t>Squad OMCM</t>
+  </si>
+  <si>
+    <t>2026-09-01</t>
+  </si>
+  <si>
     <t>Nom</t>
   </si>
   <si>
@@ -215,6 +221,12 @@
     <t>Sprint #01</t>
   </si>
   <si>
+    <t>2026-09-07</t>
+  </si>
+  <si>
+    <t>2026-09-25</t>
+  </si>
+  <si>
     <t>2026-08-17</t>
   </si>
   <si>
@@ -245,19 +257,31 @@
     <t>S1</t>
   </si>
   <si>
+    <t>2026-09-11</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>2026-09-21</t>
+  </si>
+  <si>
     <t>2026-08-21</t>
   </si>
   <si>
-    <t>S2</t>
-  </si>
-  <si>
     <t>2026-08-24</t>
   </si>
   <si>
     <t>2026-08-28</t>
-  </si>
-  <si>
-    <t>S3</t>
   </si>
   <si>
     <t>2026-08-31</t>
@@ -506,6 +530,9 @@
   </si>
   <si>
     <t>finaliser avec l’import mensuel dans le rôle exploitant, finaliser les modification types email interactions gestionnaire et les éléments manager</t>
+  </si>
+  <si>
+    <t>2026-09-01 11:15</t>
   </si>
   <si>
     <t>Frontend : finaliser avec l’import mensuel dans le rôle exploitant, finaliser les modification types email interactions gestionnaire et les éléments manager</t>
@@ -1081,7 +1108,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1105,7 +1132,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1113,7 +1140,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1129,7 +1156,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1156,7 +1183,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1195,6 +1222,23 @@
       </c>
       <c r="E2" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1220,232 +1264,232 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
         <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
         <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
         <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D7" t="s">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
         <v>53</v>
       </c>
-      <c r="B9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>51</v>
-      </c>
       <c r="E9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
         <v>16</v>
       </c>
       <c r="E10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1457,7 +1501,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1470,45 +1514,45 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E2">
         <v>3</v>
       </c>
       <c r="F2">
-        <v>564</v>
+        <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1516,13 +1560,13 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -1531,7 +1575,30 @@
         <v>564</v>
       </c>
       <c r="G3" t="s">
-        <v>27</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>564</v>
+      </c>
+      <c r="G4" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1543,7 +1610,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1558,103 +1625,103 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F2">
         <v>5</v>
       </c>
       <c r="G2">
-        <v>188</v>
+        <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F3">
         <v>5</v>
       </c>
       <c r="G3">
-        <v>188</v>
+        <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E4" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="F4">
         <v>5</v>
       </c>
       <c r="G4">
-        <v>188</v>
+        <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1662,16 +1729,16 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -1680,7 +1747,7 @@
         <v>188</v>
       </c>
       <c r="H5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1688,16 +1755,16 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D6" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E6" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F6">
         <v>5</v>
@@ -1706,7 +1773,7 @@
         <v>188</v>
       </c>
       <c r="H6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1714,16 +1781,16 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D7" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="F7">
         <v>5</v>
@@ -1732,7 +1799,85 @@
         <v>188</v>
       </c>
       <c r="H7" t="s">
-        <v>27</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+      <c r="G8">
+        <v>188</v>
+      </c>
+      <c r="H8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F9">
+        <v>5</v>
+      </c>
+      <c r="G9">
+        <v>188</v>
+      </c>
+      <c r="H9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F10">
+        <v>5</v>
+      </c>
+      <c r="G10">
+        <v>188</v>
+      </c>
+      <c r="H10" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1767,46 +1912,46 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1814,22 +1959,22 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G2" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="H2" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I2">
         <v>40</v>
@@ -1838,19 +1983,19 @@
         <v>34</v>
       </c>
       <c r="K2" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O2" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1858,22 +2003,22 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="G3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H3" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="I3">
         <v>40</v>
@@ -1882,19 +2027,19 @@
         <v>25</v>
       </c>
       <c r="K3" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O3" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1902,22 +2047,22 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="G4" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="H4" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="I4">
         <v>40</v>
@@ -1926,19 +2071,19 @@
         <v>28</v>
       </c>
       <c r="K4" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O4" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1946,22 +2091,22 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G5" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="H5" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="I5">
         <v>40</v>
@@ -1970,19 +2115,19 @@
         <v>20</v>
       </c>
       <c r="K5" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O5" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1990,22 +2135,22 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="G6" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="H6" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="I6">
         <v>17.5</v>
@@ -2014,19 +2159,19 @@
         <v>14</v>
       </c>
       <c r="K6" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="L6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O6" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -2034,22 +2179,22 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="G7" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="H7" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="I7">
         <v>40</v>
@@ -2058,19 +2203,19 @@
         <v>35</v>
       </c>
       <c r="K7" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O7" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -2078,22 +2223,22 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="G8" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="H8" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="I8">
         <v>40</v>
@@ -2102,19 +2247,19 @@
         <v>35</v>
       </c>
       <c r="K8" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="L8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O8" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -2122,22 +2267,22 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G9" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="H9" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="I9">
         <v>40</v>
@@ -2146,19 +2291,19 @@
         <v>32</v>
       </c>
       <c r="K9" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O9" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -2166,22 +2311,22 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E10" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G10" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="H10" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="I10">
         <v>40</v>
@@ -2190,19 +2335,19 @@
         <v>35</v>
       </c>
       <c r="K10" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O10" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -2210,22 +2355,22 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="G11" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="H11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="I11">
         <v>17.5</v>
@@ -2234,19 +2379,19 @@
         <v>8</v>
       </c>
       <c r="K11" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="L11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="M11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O11" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -2254,22 +2399,22 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E12" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="G12" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="H12" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="I12">
         <v>40</v>
@@ -2278,19 +2423,19 @@
         <v>35</v>
       </c>
       <c r="K12" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O12" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -2298,22 +2443,22 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E13" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G13" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H13" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="I13">
         <v>35</v>
@@ -2322,19 +2467,19 @@
         <v>34</v>
       </c>
       <c r="K13" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O13" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -2342,22 +2487,22 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E14" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G14" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H14" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="I14">
         <v>35</v>
@@ -2366,19 +2511,19 @@
         <v>33</v>
       </c>
       <c r="K14" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O14" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -2386,22 +2531,22 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="G15" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="H15" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="I15">
         <v>32</v>
@@ -2410,19 +2555,19 @@
         <v>30</v>
       </c>
       <c r="K15" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O15" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -2430,22 +2575,22 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E16" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="G16" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="H16" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="I16">
         <v>30</v>
@@ -2454,19 +2599,19 @@
         <v>31</v>
       </c>
       <c r="K16" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="L16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M16" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N16" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O16" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -2474,22 +2619,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E17" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G17" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H17" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I17">
         <v>28</v>
@@ -2498,19 +2643,19 @@
         <v>27</v>
       </c>
       <c r="K17" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L17" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M17" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N17" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O17" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -2518,22 +2663,22 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C18" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D18" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E18" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G18" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H18" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="I18">
         <v>36</v>
@@ -2542,19 +2687,19 @@
         <v>38</v>
       </c>
       <c r="K18" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="L18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M18" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N18" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O18" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -2562,22 +2707,22 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D19" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E19" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G19" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H19" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="I19">
         <v>34</v>
@@ -2586,19 +2731,19 @@
         <v>32</v>
       </c>
       <c r="K19" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="L19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M19" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N19" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O19" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
@@ -2606,22 +2751,22 @@
         <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E20" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="G20" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="H20" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="I20">
         <v>34</v>
@@ -2630,19 +2775,19 @@
         <v>35</v>
       </c>
       <c r="K20" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="L20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O20" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -2650,22 +2795,22 @@
         <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E21" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="G21" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="H21" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="I21">
         <v>32</v>
@@ -2674,19 +2819,19 @@
         <v>20</v>
       </c>
       <c r="K21" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="L21" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="M21" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N21" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O21" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -2694,22 +2839,22 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D22" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E22" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G22" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H22" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="I22">
         <v>30</v>
@@ -2718,19 +2863,19 @@
         <v>38</v>
       </c>
       <c r="K22" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L22" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M22" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N22" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O22" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -2738,22 +2883,22 @@
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D23" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E23" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G23" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H23" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I23">
         <v>34</v>
@@ -2762,19 +2907,19 @@
         <v>33</v>
       </c>
       <c r="K23" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="L23" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M23" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N23" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O23" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -2782,22 +2927,22 @@
         <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C24" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D24" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E24" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G24" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H24" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="I24">
         <v>32</v>
@@ -2806,19 +2951,19 @@
         <v>30</v>
       </c>
       <c r="K24" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="L24" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M24" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N24" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O24" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -2826,22 +2971,22 @@
         <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C25" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D25" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E25" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="G25" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="H25" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="I25">
         <v>30</v>
@@ -2850,19 +2995,19 @@
         <v>29</v>
       </c>
       <c r="K25" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="L25" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M25" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N25" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O25" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -2870,22 +3015,22 @@
         <v>16</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C26" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E26" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="G26" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="H26" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I26">
         <v>32</v>
@@ -2894,19 +3039,19 @@
         <v>12</v>
       </c>
       <c r="K26" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="L26" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="M26" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="N26" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O26" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -2914,22 +3059,22 @@
         <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C27" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D27" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E27" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G27" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H27" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="I27">
         <v>30</v>
@@ -2938,19 +3083,19 @@
         <v>28</v>
       </c>
       <c r="K27" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="L27" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M27" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N27" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O27" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -2958,43 +3103,43 @@
         <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C28" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D28" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E28" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="G28" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="H28" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="I28">
         <v>12</v>
       </c>
       <c r="J28" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K28" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="L28" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="M28" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N28" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O28" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -3002,43 +3147,43 @@
         <v>16</v>
       </c>
       <c r="B29" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C29" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D29" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E29" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="G29" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="H29" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="I29">
         <v>35</v>
       </c>
       <c r="J29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K29" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L29" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="M29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O29" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -3046,22 +3191,22 @@
         <v>16</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C30" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D30" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E30" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G30" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="H30" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="I30">
         <v>35</v>
@@ -3070,19 +3215,19 @@
         <v>30</v>
       </c>
       <c r="K30" t="s">
-        <v>101</v>
+        <v>150</v>
       </c>
       <c r="L30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M30" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N30" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O30" t="s">
-        <v>2</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -3090,43 +3235,43 @@
         <v>16</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C31" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D31" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E31" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G31" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="H31" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="I31">
         <v>35</v>
       </c>
       <c r="J31" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K31" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L31" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="M31" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N31" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O31" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -3134,43 +3279,43 @@
         <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C32" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D32" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E32" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="G32" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="H32" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="I32">
         <v>35</v>
       </c>
       <c r="J32" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K32" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="L32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="M32" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N32" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O32" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -3178,43 +3323,43 @@
         <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C33" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D33" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E33" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="G33" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="H33" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="I33">
         <v>35</v>
       </c>
       <c r="J33" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K33" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="L33" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M33" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N33" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O33" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3237,268 +3382,268 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="B2" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="C2" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D2" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="B3" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="C3" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D3" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="B4" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C4" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D4" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="B5" t="s">
+        <v>194</v>
+      </c>
+      <c r="C5" t="s">
         <v>185</v>
       </c>
-      <c r="C5" t="s">
-        <v>176</v>
-      </c>
       <c r="D5" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="B6" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="C6" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D6" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="B7" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="C7" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D7" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B8" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="C8" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D8" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="B9" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="C9" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D9" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="B10" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C10" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D10" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="B11" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="C11" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D11" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="B12" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="C12" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D12" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="B13" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C13" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D13" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="B14" t="s">
+        <v>194</v>
+      </c>
+      <c r="C14" t="s">
         <v>185</v>
       </c>
-      <c r="C14" t="s">
-        <v>176</v>
-      </c>
       <c r="D14" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="B15" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="C15" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D15" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="B16" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="C16" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D16" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="B17" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="C17" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D17" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="B18" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="C18" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D18" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="B19" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C19" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D19" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -3521,19 +3666,19 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bd : déclaration d’un congé
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="222">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,127 +26,130 @@
     <t>Généré le</t>
   </si>
   <si>
+    <t>2026-09-04 12:38</t>
+  </si>
+  <si>
+    <t>Squads</t>
+  </si>
+  <si>
+    <t>Comptes utilisateurs</t>
+  </si>
+  <si>
+    <t>dont actifs</t>
+  </si>
+  <si>
+    <t>Sprints</t>
+  </si>
+  <si>
+    <t>Semaines de revue</t>
+  </si>
+  <si>
+    <t>Objectifs saisis</t>
+  </si>
+  <si>
+    <t>dont validés</t>
+  </si>
+  <si>
+    <t>Jours fériés enregistrés</t>
+  </si>
+  <si>
+    <t>Congés enregistrés</t>
+  </si>
+  <si>
+    <t>Squad</t>
+  </si>
+  <si>
+    <t>Heures / jour</t>
+  </si>
+  <si>
+    <t>Membres</t>
+  </si>
+  <si>
+    <t>Créée le</t>
+  </si>
+  <si>
+    <t>Squad Digital</t>
+  </si>
+  <si>
+    <t>2026-08-20</t>
+  </si>
+  <si>
+    <t>Squad OMCM</t>
+  </si>
+  <si>
+    <t>2026-09-01</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Rôle</t>
+  </si>
+  <si>
+    <t>Actif</t>
+  </si>
+  <si>
+    <t>Mot de passe à changer</t>
+  </si>
+  <si>
+    <t>Dernière connexion</t>
+  </si>
+  <si>
+    <t>BELINGA Yan</t>
+  </si>
+  <si>
+    <t>yan.belinga@orange.com</t>
+  </si>
+  <si>
+    <t>Développeur</t>
+  </si>
+  <si>
+    <t>oui</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>2026-08-25 15:41</t>
+  </si>
+  <si>
+    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
+  </si>
+  <si>
+    <t>charlene.djoungang@orange.com</t>
+  </si>
+  <si>
+    <t>Observateur</t>
+  </si>
+  <si>
+    <t>2026-08-25 08:50</t>
+  </si>
+  <si>
+    <t>FOGUE Hervé</t>
+  </si>
+  <si>
+    <t>herve.soubgui@orange.com</t>
+  </si>
+  <si>
+    <t>Tech Lead</t>
+  </si>
+  <si>
+    <t>2026-08-20 08:35</t>
+  </si>
+  <si>
+    <t>FOKA Emmanuel</t>
+  </si>
+  <si>
+    <t>emmanuel.foka@orange.com</t>
+  </si>
+  <si>
+    <t>Scrum Master</t>
+  </si>
+  <si>
     <t>2026-09-04 07:49</t>
-  </si>
-  <si>
-    <t>Squads</t>
-  </si>
-  <si>
-    <t>Comptes utilisateurs</t>
-  </si>
-  <si>
-    <t>dont actifs</t>
-  </si>
-  <si>
-    <t>Sprints</t>
-  </si>
-  <si>
-    <t>Semaines de revue</t>
-  </si>
-  <si>
-    <t>Objectifs saisis</t>
-  </si>
-  <si>
-    <t>dont validés</t>
-  </si>
-  <si>
-    <t>Jours fériés enregistrés</t>
-  </si>
-  <si>
-    <t>Congés enregistrés</t>
-  </si>
-  <si>
-    <t>Squad</t>
-  </si>
-  <si>
-    <t>Heures / jour</t>
-  </si>
-  <si>
-    <t>Membres</t>
-  </si>
-  <si>
-    <t>Créée le</t>
-  </si>
-  <si>
-    <t>Squad Digital</t>
-  </si>
-  <si>
-    <t>2026-08-20</t>
-  </si>
-  <si>
-    <t>Squad OMCM</t>
-  </si>
-  <si>
-    <t>2026-09-01</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Rôle</t>
-  </si>
-  <si>
-    <t>Actif</t>
-  </si>
-  <si>
-    <t>Mot de passe à changer</t>
-  </si>
-  <si>
-    <t>Dernière connexion</t>
-  </si>
-  <si>
-    <t>BELINGA Yan</t>
-  </si>
-  <si>
-    <t>yan.belinga@orange.com</t>
-  </si>
-  <si>
-    <t>Développeur</t>
-  </si>
-  <si>
-    <t>oui</t>
-  </si>
-  <si>
-    <t>non</t>
-  </si>
-  <si>
-    <t>2026-08-25 15:41</t>
-  </si>
-  <si>
-    <t>DJOUNGANG Charlène Ext O-CM/DEC</t>
-  </si>
-  <si>
-    <t>charlene.djoungang@orange.com</t>
-  </si>
-  <si>
-    <t>Observateur</t>
-  </si>
-  <si>
-    <t>2026-08-25 08:50</t>
-  </si>
-  <si>
-    <t>FOGUE Hervé</t>
-  </si>
-  <si>
-    <t>herve.soubgui@orange.com</t>
-  </si>
-  <si>
-    <t>Tech Lead</t>
-  </si>
-  <si>
-    <t>2026-08-20 08:35</t>
-  </si>
-  <si>
-    <t>FOKA Emmanuel</t>
-  </si>
-  <si>
-    <t>emmanuel.foka@orange.com</t>
-  </si>
-  <si>
-    <t>Scrum Master</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -523,15 +526,12 @@
     <t>déploiement GTR Flow en preprod</t>
   </si>
   <si>
-    <t>2026-08-31 08:18</t>
+    <t>2026-09-04 09:38</t>
   </si>
   <si>
     <t>finaliser avec l’import mensuel dans le rôle exploitant, finaliser les modification types email interactions gestionnaire et les éléments manager</t>
   </si>
   <si>
-    <t>2026-09-01 11:15</t>
-  </si>
-  <si>
     <t>Frontend : finaliser avec l’import mensuel dans le rôle exploitant, finaliser les modification types email interactions gestionnaire et les éléments manager</t>
   </si>
   <si>
@@ -683,6 +683,9 @@
   </si>
   <si>
     <t>Motif</t>
+  </si>
+  <si>
+    <t>Soucis personnel</t>
   </si>
 </sst>
 </file>
@@ -1172,7 +1175,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1374,15 +1377,15 @@
         <v>30</v>
       </c>
       <c r="G5" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
         <v>28</v>
@@ -1397,15 +1400,15 @@
         <v>29</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
         <v>28</v>
@@ -1420,21 +1423,21 @@
         <v>29</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
         <v>29</v>
@@ -1443,21 +1446,21 @@
         <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
         <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E9" t="s">
         <v>29</v>
@@ -1466,15 +1469,15 @@
         <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
         <v>28</v>
@@ -1489,7 +1492,7 @@
         <v>29</v>
       </c>
       <c r="G10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1514,22 +1517,22 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1537,13 +1540,13 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -1560,13 +1563,13 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -1583,13 +1586,13 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -1625,25 +1628,25 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1651,16 +1654,16 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F2">
         <v>5</v>
@@ -1677,16 +1680,16 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -1703,16 +1706,16 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F4">
         <v>5</v>
@@ -1729,16 +1732,16 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -1755,16 +1758,16 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F6">
         <v>5</v>
@@ -1781,16 +1784,16 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F7">
         <v>5</v>
@@ -1807,16 +1810,16 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F8">
         <v>5</v>
@@ -1833,16 +1836,16 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F9">
         <v>5</v>
@@ -1859,16 +1862,16 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F10">
         <v>5</v>
@@ -1912,46 +1915,46 @@
         <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1959,22 +1962,22 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I2">
         <v>40</v>
@@ -1983,19 +1986,19 @@
         <v>34</v>
       </c>
       <c r="K2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L2" t="s">
         <v>29</v>
       </c>
       <c r="M2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -2003,22 +2006,22 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D3" t="s">
         <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G3" t="s">
         <v>38</v>
       </c>
       <c r="H3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I3">
         <v>40</v>
@@ -2027,19 +2030,19 @@
         <v>25</v>
       </c>
       <c r="K3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L3" t="s">
         <v>29</v>
       </c>
       <c r="M3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -2047,22 +2050,22 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I4">
         <v>40</v>
@@ -2071,19 +2074,19 @@
         <v>28</v>
       </c>
       <c r="K4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L4" t="s">
         <v>29</v>
       </c>
       <c r="M4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -2091,22 +2094,22 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I5">
         <v>40</v>
@@ -2115,19 +2118,19 @@
         <v>20</v>
       </c>
       <c r="K5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L5" t="s">
         <v>29</v>
       </c>
       <c r="M5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -2135,22 +2138,22 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I6">
         <v>17.5</v>
@@ -2159,19 +2162,19 @@
         <v>14</v>
       </c>
       <c r="K6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="L6" t="s">
         <v>29</v>
       </c>
       <c r="M6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -2179,22 +2182,22 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
         <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I7">
         <v>40</v>
@@ -2203,19 +2206,19 @@
         <v>35</v>
       </c>
       <c r="K7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L7" t="s">
         <v>29</v>
       </c>
       <c r="M7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -2223,22 +2226,22 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I8">
         <v>40</v>
@@ -2247,19 +2250,19 @@
         <v>35</v>
       </c>
       <c r="K8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L8" t="s">
         <v>29</v>
       </c>
       <c r="M8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -2267,22 +2270,22 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I9">
         <v>40</v>
@@ -2291,19 +2294,19 @@
         <v>32</v>
       </c>
       <c r="K9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L9" t="s">
         <v>29</v>
       </c>
       <c r="M9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -2311,22 +2314,22 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D10" t="s">
         <v>26</v>
       </c>
       <c r="E10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I10">
         <v>40</v>
@@ -2335,19 +2338,19 @@
         <v>35</v>
       </c>
       <c r="K10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L10" t="s">
         <v>29</v>
       </c>
       <c r="M10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -2355,22 +2358,22 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I11">
         <v>17.5</v>
@@ -2379,19 +2382,19 @@
         <v>8</v>
       </c>
       <c r="K11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="L11" t="s">
         <v>30</v>
       </c>
       <c r="M11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -2399,22 +2402,22 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D12" t="s">
         <v>40</v>
       </c>
       <c r="E12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H12" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I12">
         <v>40</v>
@@ -2423,19 +2426,19 @@
         <v>35</v>
       </c>
       <c r="K12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L12" t="s">
         <v>29</v>
       </c>
       <c r="M12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -2443,22 +2446,22 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I13">
         <v>35</v>
@@ -2467,19 +2470,19 @@
         <v>34</v>
       </c>
       <c r="K13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L13" t="s">
         <v>29</v>
       </c>
       <c r="M13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -2487,22 +2490,22 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
         <v>26</v>
       </c>
       <c r="E14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I14">
         <v>35</v>
@@ -2511,19 +2514,19 @@
         <v>33</v>
       </c>
       <c r="K14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L14" t="s">
         <v>29</v>
       </c>
       <c r="M14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -2531,22 +2534,22 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H15" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I15">
         <v>32</v>
@@ -2555,19 +2558,19 @@
         <v>30</v>
       </c>
       <c r="K15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L15" t="s">
         <v>29</v>
       </c>
       <c r="M15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -2575,22 +2578,22 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G16" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I16">
         <v>30</v>
@@ -2599,19 +2602,19 @@
         <v>31</v>
       </c>
       <c r="K16" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="L16" t="s">
         <v>29</v>
       </c>
       <c r="M16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O16" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -2619,22 +2622,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D17" t="s">
         <v>36</v>
       </c>
       <c r="E17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H17" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I17">
         <v>28</v>
@@ -2643,19 +2646,19 @@
         <v>27</v>
       </c>
       <c r="K17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L17" t="s">
         <v>29</v>
       </c>
       <c r="M17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O17" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -2663,22 +2666,22 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G18" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I18">
         <v>36</v>
@@ -2687,19 +2690,19 @@
         <v>38</v>
       </c>
       <c r="K18" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L18" t="s">
         <v>29</v>
       </c>
       <c r="M18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O18" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -2707,22 +2710,22 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D19" t="s">
         <v>26</v>
       </c>
       <c r="E19" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G19" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H19" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I19">
         <v>34</v>
@@ -2731,19 +2734,19 @@
         <v>32</v>
       </c>
       <c r="K19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L19" t="s">
         <v>29</v>
       </c>
       <c r="M19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O19" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
@@ -2751,22 +2754,22 @@
         <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D20" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G20" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H20" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I20">
         <v>34</v>
@@ -2775,19 +2778,19 @@
         <v>35</v>
       </c>
       <c r="K20" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="L20" t="s">
         <v>29</v>
       </c>
       <c r="M20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O20" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -2795,22 +2798,22 @@
         <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C21" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D21" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G21" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H21" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I21">
         <v>32</v>
@@ -2819,19 +2822,19 @@
         <v>20</v>
       </c>
       <c r="K21" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="L21" t="s">
         <v>30</v>
       </c>
       <c r="M21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O21" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -2839,22 +2842,22 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D22" t="s">
         <v>36</v>
       </c>
       <c r="E22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H22" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I22">
         <v>30</v>
@@ -2863,19 +2866,19 @@
         <v>38</v>
       </c>
       <c r="K22" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L22" t="s">
         <v>29</v>
       </c>
       <c r="M22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -2883,22 +2886,22 @@
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D23" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H23" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I23">
         <v>34</v>
@@ -2907,19 +2910,19 @@
         <v>33</v>
       </c>
       <c r="K23" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="L23" t="s">
         <v>29</v>
       </c>
       <c r="M23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O23" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -2927,22 +2930,22 @@
         <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C24" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
       </c>
       <c r="E24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G24" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H24" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I24">
         <v>32</v>
@@ -2951,19 +2954,19 @@
         <v>30</v>
       </c>
       <c r="K24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L24" t="s">
         <v>29</v>
       </c>
       <c r="M24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O24" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -2971,22 +2974,22 @@
         <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C25" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D25" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E25" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G25" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H25" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I25">
         <v>30</v>
@@ -2995,19 +2998,19 @@
         <v>29</v>
       </c>
       <c r="K25" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="L25" t="s">
         <v>29</v>
       </c>
       <c r="M25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O25" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -3015,22 +3018,22 @@
         <v>16</v>
       </c>
       <c r="B26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C26" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G26" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I26">
         <v>32</v>
@@ -3039,19 +3042,19 @@
         <v>12</v>
       </c>
       <c r="K26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="L26" t="s">
         <v>30</v>
       </c>
       <c r="M26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -3059,22 +3062,22 @@
         <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C27" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D27" t="s">
         <v>36</v>
       </c>
       <c r="E27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H27" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I27">
         <v>30</v>
@@ -3083,19 +3086,19 @@
         <v>28</v>
       </c>
       <c r="K27" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="L27" t="s">
         <v>29</v>
       </c>
       <c r="M27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O27" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -3103,43 +3106,43 @@
         <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C28" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D28" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E28" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H28" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I28">
         <v>12</v>
       </c>
       <c r="J28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L28" t="s">
         <v>30</v>
       </c>
       <c r="M28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O28" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -3147,43 +3150,43 @@
         <v>16</v>
       </c>
       <c r="B29" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C29" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D29" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G29" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H29" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I29">
         <v>35</v>
       </c>
-      <c r="J29" t="s">
-        <v>45</v>
+      <c r="J29">
+        <v>32</v>
       </c>
       <c r="K29" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L29" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M29" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N29" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O29" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -3191,22 +3194,22 @@
         <v>16</v>
       </c>
       <c r="B30" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C30" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D30" t="s">
         <v>26</v>
       </c>
       <c r="E30" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G30" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H30" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I30">
         <v>35</v>
@@ -3215,19 +3218,19 @@
         <v>30</v>
       </c>
       <c r="K30" t="s">
-        <v>149</v>
+        <v>109</v>
       </c>
       <c r="L30" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O30" t="s">
-        <v>169</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -3235,19 +3238,19 @@
         <v>16</v>
       </c>
       <c r="B31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C31" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D31" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G31" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H31" t="s">
         <v>170</v>
@@ -3256,19 +3259,19 @@
         <v>35</v>
       </c>
       <c r="J31" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K31" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L31" t="s">
         <v>30</v>
       </c>
       <c r="M31" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N31" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O31" t="s">
         <v>171</v>
@@ -3279,16 +3282,16 @@
         <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C32" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D32" t="s">
         <v>36</v>
       </c>
       <c r="E32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G32" t="s">
         <v>172</v>
@@ -3300,19 +3303,19 @@
         <v>35</v>
       </c>
       <c r="J32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L32" t="s">
         <v>30</v>
       </c>
       <c r="M32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O32" t="s">
         <v>174</v>
@@ -3323,16 +3326,16 @@
         <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C33" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D33" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E33" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G33" t="s">
         <v>175</v>
@@ -3344,19 +3347,19 @@
         <v>35</v>
       </c>
       <c r="J33" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L33" t="s">
         <v>29</v>
       </c>
       <c r="M33" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N33" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O33" t="s">
         <v>177</v>
@@ -3367,22 +3370,22 @@
         <v>16</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C34" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D34" t="s">
         <v>40</v>
       </c>
       <c r="E34" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G34" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H34" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I34">
         <v>35</v>
@@ -3391,16 +3394,16 @@
         <v>30</v>
       </c>
       <c r="K34" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L34" t="s">
         <v>30</v>
       </c>
       <c r="M34" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N34" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O34" t="s">
         <v>178</v>
@@ -3699,7 +3702,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -3725,6 +3728,23 @@
         <v>220</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" t="s">
+        <v>221</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
bd : modification d’un sprint
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="221">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-09-04 15:24</t>
+    <t>2026-09-07 08:47</t>
   </si>
   <si>
     <t>Squads</t>
@@ -149,7 +149,7 @@
     <t>Scrum Master</t>
   </si>
   <si>
-    <t>2026-09-04 07:49</t>
+    <t>2026-09-07 08:45</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -532,7 +532,7 @@
     <t>finaliser avec l’import mensuel dans le rôle exploitant, finaliser les modification types email interactions gestionnaire et les éléments manager</t>
   </si>
   <si>
-    <t>2026-09-04 14:24</t>
+    <t>2026-09-04 15:24</t>
   </si>
   <si>
     <t>Frontend : finaliser avec l’import mensuel dans le rôle exploitant, finaliser les modification types email interactions gestionnaire et les éléments manager</t>
@@ -545,9 +545,6 @@
   </si>
   <si>
     <t>supervision que les points soient bouclés : compteur des clics, CxRecov, GTR Flow, analyse des points sur le prochain sprint</t>
-  </si>
-  <si>
-    <t>2026-08-31 08:23</t>
   </si>
   <si>
     <t>Compteurs des Clics</t>
@@ -1159,7 +1156,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1578,7 +1575,7 @@
         <v>556</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1802,7 +1799,7 @@
         <v>180</v>
       </c>
       <c r="H7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -3221,7 +3218,7 @@
         <v>109</v>
       </c>
       <c r="L30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M30" t="s">
         <v>46</v>
@@ -3302,14 +3299,14 @@
       <c r="I32">
         <v>35</v>
       </c>
-      <c r="J32" t="s">
-        <v>46</v>
+      <c r="J32">
+        <v>35</v>
       </c>
       <c r="K32" t="s">
         <v>109</v>
       </c>
       <c r="L32" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M32" t="s">
         <v>46</v>
@@ -3318,7 +3315,7 @@
         <v>46</v>
       </c>
       <c r="O32" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -3338,10 +3335,10 @@
         <v>114</v>
       </c>
       <c r="G33" t="s">
+        <v>175</v>
+      </c>
+      <c r="H33" t="s">
         <v>176</v>
-      </c>
-      <c r="H33" t="s">
-        <v>177</v>
       </c>
       <c r="I33">
         <v>35</v>
@@ -3362,7 +3359,7 @@
         <v>46</v>
       </c>
       <c r="O33" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -3385,268 +3382,268 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>181</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" t="s">
         <v>183</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>184</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>185</v>
-      </c>
-      <c r="D2" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B3" t="s">
         <v>187</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D3" t="s">
         <v>188</v>
-      </c>
-      <c r="C3" t="s">
-        <v>185</v>
-      </c>
-      <c r="D3" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B4" t="s">
         <v>190</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D4" t="s">
         <v>191</v>
-      </c>
-      <c r="C4" t="s">
-        <v>185</v>
-      </c>
-      <c r="D4" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>192</v>
+      </c>
+      <c r="B5" t="s">
         <v>193</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D5" t="s">
         <v>194</v>
-      </c>
-      <c r="C5" t="s">
-        <v>185</v>
-      </c>
-      <c r="D5" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B6" t="s">
         <v>196</v>
       </c>
-      <c r="B6" t="s">
-        <v>197</v>
-      </c>
       <c r="C6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" t="s">
         <v>198</v>
       </c>
-      <c r="B7" t="s">
-        <v>199</v>
-      </c>
       <c r="C7" t="s">
+        <v>184</v>
+      </c>
+      <c r="D7" t="s">
         <v>185</v>
-      </c>
-      <c r="D7" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B8" t="s">
         <v>200</v>
       </c>
-      <c r="B8" t="s">
-        <v>201</v>
-      </c>
       <c r="C8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>201</v>
+      </c>
+      <c r="B9" t="s">
         <v>202</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>184</v>
+      </c>
+      <c r="D9" t="s">
         <v>203</v>
-      </c>
-      <c r="C9" t="s">
-        <v>185</v>
-      </c>
-      <c r="D9" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>204</v>
+      </c>
+      <c r="B10" t="s">
         <v>205</v>
       </c>
-      <c r="B10" t="s">
-        <v>206</v>
-      </c>
       <c r="C10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B11" t="s">
+        <v>183</v>
+      </c>
+      <c r="C11" t="s">
         <v>184</v>
       </c>
-      <c r="C11" t="s">
-        <v>185</v>
-      </c>
       <c r="D11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C12" t="s">
+        <v>184</v>
+      </c>
+      <c r="D12" t="s">
         <v>185</v>
-      </c>
-      <c r="D12" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B13" t="s">
+        <v>190</v>
+      </c>
+      <c r="C13" t="s">
+        <v>184</v>
+      </c>
+      <c r="D13" t="s">
         <v>191</v>
-      </c>
-      <c r="C13" t="s">
-        <v>185</v>
-      </c>
-      <c r="D13" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B14" t="s">
+        <v>193</v>
+      </c>
+      <c r="C14" t="s">
+        <v>184</v>
+      </c>
+      <c r="D14" t="s">
         <v>194</v>
-      </c>
-      <c r="C14" t="s">
-        <v>185</v>
-      </c>
-      <c r="D14" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B16" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C16" t="s">
+        <v>184</v>
+      </c>
+      <c r="D16" t="s">
         <v>185</v>
-      </c>
-      <c r="D16" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C17" t="s">
+        <v>184</v>
+      </c>
+      <c r="D17" t="s">
         <v>185</v>
-      </c>
-      <c r="D17" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>213</v>
+      </c>
+      <c r="B18" t="s">
+        <v>202</v>
+      </c>
+      <c r="C18" t="s">
+        <v>184</v>
+      </c>
+      <c r="D18" t="s">
         <v>214</v>
-      </c>
-      <c r="B18" t="s">
-        <v>203</v>
-      </c>
-      <c r="C18" t="s">
-        <v>185</v>
-      </c>
-      <c r="D18" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C19" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D19" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -3669,19 +3666,19 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>219</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3698,7 +3695,7 @@
         <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bd : suppression d'un sprint (force=true)
</commit_message>
<xml_diff>
--- a/bd/sprint-tracker.xlsx
+++ b/bd/sprint-tracker.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="215">
   <si>
     <t>Sprint Tracker — export de la base</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Généré le</t>
   </si>
   <si>
-    <t>2026-09-07 15:46</t>
+    <t>2026-09-10 13:52</t>
   </si>
   <si>
     <t>Squads</t>
@@ -149,7 +149,7 @@
     <t>Scrum Master</t>
   </si>
   <si>
-    <t>2026-09-07 08:45</t>
+    <t>2026-09-10 13:42</t>
   </si>
   <si>
     <t>MBENG Ivan</t>
@@ -182,7 +182,7 @@
     <t>—</t>
   </si>
   <si>
-    <t>2026-09-07 14:55</t>
+    <t>2026-09-10 13:48</t>
   </si>
   <si>
     <t>Test User</t>
@@ -218,15 +218,6 @@
     <t>Clôturé</t>
   </si>
   <si>
-    <t>Sprint #02</t>
-  </si>
-  <si>
-    <t>2026-09-14</t>
-  </si>
-  <si>
-    <t>2026-10-02</t>
-  </si>
-  <si>
     <t>Sprint #01</t>
   </si>
   <si>
@@ -260,31 +251,19 @@
     <t>S1</t>
   </si>
   <si>
-    <t>2026-09-18</t>
+    <t>2026-08-21</t>
   </si>
   <si>
     <t>S2</t>
   </si>
   <si>
-    <t>2026-09-21</t>
-  </si>
-  <si>
-    <t>2026-09-25</t>
+    <t>2026-08-24</t>
+  </si>
+  <si>
+    <t>2026-08-28</t>
   </si>
   <si>
     <t>S3</t>
-  </si>
-  <si>
-    <t>2026-09-28</t>
-  </si>
-  <si>
-    <t>2026-08-21</t>
-  </si>
-  <si>
-    <t>2026-08-24</t>
-  </si>
-  <si>
-    <t>2026-08-28</t>
   </si>
   <si>
     <t>2026-08-31</t>
@@ -1135,7 +1114,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1143,7 +1122,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1221,7 +1200,7 @@
         <v>7</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -1504,7 +1483,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1552,10 +1531,10 @@
         <v>3</v>
       </c>
       <c r="F2">
-        <v>564</v>
+        <v>556</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1575,32 +1554,9 @@
         <v>3</v>
       </c>
       <c r="F3">
-        <v>556</v>
+        <v>564</v>
       </c>
       <c r="G3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D4" t="s">
-        <v>74</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4">
-        <v>564</v>
-      </c>
-      <c r="G4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1613,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1631,22 +1587,22 @@
         <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>64</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1657,13 +1613,13 @@
         <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D2" t="s">
         <v>67</v>
       </c>
       <c r="E2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F2">
         <v>5</v>
@@ -1672,7 +1628,7 @@
         <v>188</v>
       </c>
       <c r="H2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1683,13 +1639,13 @@
         <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -1698,7 +1654,7 @@
         <v>188</v>
       </c>
       <c r="H3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1709,22 +1665,22 @@
         <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="F4">
         <v>5</v>
       </c>
       <c r="G4">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="H4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1735,13 +1691,13 @@
         <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
         <v>70</v>
       </c>
       <c r="E5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -1761,13 +1717,13 @@
         <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F6">
         <v>5</v>
@@ -1787,99 +1743,21 @@
         <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E7" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="F7">
         <v>5</v>
       </c>
       <c r="G7">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="H7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" t="s">
-        <v>79</v>
-      </c>
-      <c r="D8" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" t="s">
-        <v>91</v>
-      </c>
-      <c r="F8">
-        <v>5</v>
-      </c>
-      <c r="G8">
-        <v>188</v>
-      </c>
-      <c r="H8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" t="s">
-        <v>92</v>
-      </c>
-      <c r="E9" t="s">
-        <v>93</v>
-      </c>
-      <c r="F9">
-        <v>5</v>
-      </c>
-      <c r="G9">
-        <v>188</v>
-      </c>
-      <c r="H9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C10" t="s">
-        <v>84</v>
-      </c>
-      <c r="D10" t="s">
-        <v>94</v>
-      </c>
-      <c r="E10" t="s">
-        <v>74</v>
-      </c>
-      <c r="F10">
-        <v>5</v>
-      </c>
-      <c r="G10">
-        <v>188</v>
-      </c>
-      <c r="H10" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1918,43 +1796,43 @@
         <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1962,22 +1840,22 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G2" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="H2" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="I2">
         <v>40</v>
@@ -1986,7 +1864,7 @@
         <v>34</v>
       </c>
       <c r="K2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L2" t="s">
         <v>29</v>
@@ -1998,7 +1876,7 @@
         <v>46</v>
       </c>
       <c r="O2" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -2006,22 +1884,22 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
         <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="G3" t="s">
         <v>38</v>
       </c>
       <c r="H3" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="I3">
         <v>40</v>
@@ -2030,7 +1908,7 @@
         <v>25</v>
       </c>
       <c r="K3" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L3" t="s">
         <v>29</v>
@@ -2042,7 +1920,7 @@
         <v>46</v>
       </c>
       <c r="O3" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -2050,22 +1928,22 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
         <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="G4" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="H4" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="I4">
         <v>40</v>
@@ -2074,7 +1952,7 @@
         <v>28</v>
       </c>
       <c r="K4" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L4" t="s">
         <v>29</v>
@@ -2086,7 +1964,7 @@
         <v>46</v>
       </c>
       <c r="O4" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -2094,22 +1972,22 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
         <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="H5" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="I5">
         <v>40</v>
@@ -2118,7 +1996,7 @@
         <v>20</v>
       </c>
       <c r="K5" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L5" t="s">
         <v>29</v>
@@ -2130,7 +2008,7 @@
         <v>46</v>
       </c>
       <c r="O5" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -2138,22 +2016,22 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
         <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="G6" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="H6" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="I6">
         <v>17.5</v>
@@ -2162,7 +2040,7 @@
         <v>14</v>
       </c>
       <c r="K6" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="L6" t="s">
         <v>29</v>
@@ -2174,7 +2052,7 @@
         <v>46</v>
       </c>
       <c r="O6" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -2182,22 +2060,22 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
         <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="G7" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="H7" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="I7">
         <v>40</v>
@@ -2206,7 +2084,7 @@
         <v>35</v>
       </c>
       <c r="K7" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L7" t="s">
         <v>29</v>
@@ -2218,7 +2096,7 @@
         <v>46</v>
       </c>
       <c r="O7" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -2226,22 +2104,22 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D8" t="s">
         <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="G8" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="H8" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="I8">
         <v>40</v>
@@ -2250,7 +2128,7 @@
         <v>35</v>
       </c>
       <c r="K8" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="L8" t="s">
         <v>29</v>
@@ -2262,7 +2140,7 @@
         <v>46</v>
       </c>
       <c r="O8" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -2270,22 +2148,22 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D9" t="s">
         <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G9" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="H9" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="I9">
         <v>40</v>
@@ -2294,7 +2172,7 @@
         <v>32</v>
       </c>
       <c r="K9" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L9" t="s">
         <v>29</v>
@@ -2306,7 +2184,7 @@
         <v>46</v>
       </c>
       <c r="O9" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -2314,22 +2192,22 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D10" t="s">
         <v>26</v>
       </c>
       <c r="E10" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G10" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="H10" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="I10">
         <v>40</v>
@@ -2338,7 +2216,7 @@
         <v>35</v>
       </c>
       <c r="K10" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L10" t="s">
         <v>29</v>
@@ -2350,7 +2228,7 @@
         <v>46</v>
       </c>
       <c r="O10" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -2358,22 +2236,22 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D11" t="s">
         <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="G11" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="H11" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="I11">
         <v>17.5</v>
@@ -2382,7 +2260,7 @@
         <v>8</v>
       </c>
       <c r="K11" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="L11" t="s">
         <v>30</v>
@@ -2394,7 +2272,7 @@
         <v>46</v>
       </c>
       <c r="O11" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -2402,22 +2280,22 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D12" t="s">
         <v>40</v>
       </c>
       <c r="E12" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="G12" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="H12" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="I12">
         <v>40</v>
@@ -2426,7 +2304,7 @@
         <v>35</v>
       </c>
       <c r="K12" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L12" t="s">
         <v>29</v>
@@ -2438,7 +2316,7 @@
         <v>46</v>
       </c>
       <c r="O12" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -2446,22 +2324,22 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D13" t="s">
         <v>47</v>
       </c>
       <c r="E13" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G13" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="H13" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="I13">
         <v>35</v>
@@ -2470,7 +2348,7 @@
         <v>34</v>
       </c>
       <c r="K13" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L13" t="s">
         <v>29</v>
@@ -2482,7 +2360,7 @@
         <v>46</v>
       </c>
       <c r="O13" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -2490,22 +2368,22 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D14" t="s">
         <v>26</v>
       </c>
       <c r="E14" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G14" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="H14" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="I14">
         <v>35</v>
@@ -2514,7 +2392,7 @@
         <v>33</v>
       </c>
       <c r="K14" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L14" t="s">
         <v>29</v>
@@ -2526,7 +2404,7 @@
         <v>46</v>
       </c>
       <c r="O14" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -2534,22 +2412,22 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C15" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D15" t="s">
         <v>44</v>
       </c>
       <c r="E15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="G15" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="H15" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="I15">
         <v>32</v>
@@ -2558,7 +2436,7 @@
         <v>30</v>
       </c>
       <c r="K15" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L15" t="s">
         <v>29</v>
@@ -2570,7 +2448,7 @@
         <v>46</v>
       </c>
       <c r="O15" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -2578,22 +2456,22 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D16" t="s">
         <v>57</v>
       </c>
       <c r="E16" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="G16" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="H16" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="I16">
         <v>30</v>
@@ -2602,7 +2480,7 @@
         <v>31</v>
       </c>
       <c r="K16" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="L16" t="s">
         <v>29</v>
@@ -2614,7 +2492,7 @@
         <v>46</v>
       </c>
       <c r="O16" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -2622,22 +2500,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D17" t="s">
         <v>36</v>
       </c>
       <c r="E17" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G17" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="H17" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="I17">
         <v>28</v>
@@ -2646,7 +2524,7 @@
         <v>27</v>
       </c>
       <c r="K17" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L17" t="s">
         <v>29</v>
@@ -2658,7 +2536,7 @@
         <v>46</v>
       </c>
       <c r="O17" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -2666,22 +2544,22 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D18" t="s">
         <v>47</v>
       </c>
       <c r="E18" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G18" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="H18" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="I18">
         <v>36</v>
@@ -2690,7 +2568,7 @@
         <v>38</v>
       </c>
       <c r="K18" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="L18" t="s">
         <v>29</v>
@@ -2702,7 +2580,7 @@
         <v>46</v>
       </c>
       <c r="O18" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -2710,22 +2588,22 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D19" t="s">
         <v>26</v>
       </c>
       <c r="E19" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G19" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="H19" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="I19">
         <v>34</v>
@@ -2734,7 +2612,7 @@
         <v>32</v>
       </c>
       <c r="K19" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="L19" t="s">
         <v>29</v>
@@ -2746,7 +2624,7 @@
         <v>46</v>
       </c>
       <c r="O19" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
@@ -2754,22 +2632,22 @@
         <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D20" t="s">
         <v>44</v>
       </c>
       <c r="E20" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="G20" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="H20" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="I20">
         <v>34</v>
@@ -2778,7 +2656,7 @@
         <v>35</v>
       </c>
       <c r="K20" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="L20" t="s">
         <v>29</v>
@@ -2790,7 +2668,7 @@
         <v>46</v>
       </c>
       <c r="O20" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -2798,22 +2676,22 @@
         <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D21" t="s">
         <v>57</v>
       </c>
       <c r="E21" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="G21" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="H21" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="I21">
         <v>32</v>
@@ -2822,7 +2700,7 @@
         <v>20</v>
       </c>
       <c r="K21" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="L21" t="s">
         <v>30</v>
@@ -2834,7 +2712,7 @@
         <v>46</v>
       </c>
       <c r="O21" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -2842,22 +2720,22 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C22" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D22" t="s">
         <v>36</v>
       </c>
       <c r="E22" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G22" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="H22" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="I22">
         <v>30</v>
@@ -2866,7 +2744,7 @@
         <v>38</v>
       </c>
       <c r="K22" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L22" t="s">
         <v>29</v>
@@ -2878,7 +2756,7 @@
         <v>46</v>
       </c>
       <c r="O22" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -2886,22 +2764,22 @@
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D23" t="s">
         <v>47</v>
       </c>
       <c r="E23" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G23" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="H23" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="I23">
         <v>34</v>
@@ -2910,7 +2788,7 @@
         <v>33</v>
       </c>
       <c r="K23" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="L23" t="s">
         <v>29</v>
@@ -2922,7 +2800,7 @@
         <v>46</v>
       </c>
       <c r="O23" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -2930,22 +2808,22 @@
         <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
       </c>
       <c r="E24" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G24" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="H24" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="I24">
         <v>32</v>
@@ -2954,7 +2832,7 @@
         <v>30</v>
       </c>
       <c r="K24" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="L24" t="s">
         <v>29</v>
@@ -2966,7 +2844,7 @@
         <v>46</v>
       </c>
       <c r="O24" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -2974,22 +2852,22 @@
         <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C25" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D25" t="s">
         <v>44</v>
       </c>
       <c r="E25" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="G25" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="H25" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="I25">
         <v>30</v>
@@ -2998,7 +2876,7 @@
         <v>29</v>
       </c>
       <c r="K25" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="L25" t="s">
         <v>29</v>
@@ -3010,7 +2888,7 @@
         <v>46</v>
       </c>
       <c r="O25" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -3018,22 +2896,22 @@
         <v>16</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C26" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D26" t="s">
         <v>57</v>
       </c>
       <c r="E26" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="G26" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="H26" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="I26">
         <v>32</v>
@@ -3042,19 +2920,19 @@
         <v>12</v>
       </c>
       <c r="K26" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="L26" t="s">
         <v>30</v>
       </c>
       <c r="M26" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="N26" t="s">
         <v>46</v>
       </c>
       <c r="O26" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -3062,22 +2940,22 @@
         <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D27" t="s">
         <v>36</v>
       </c>
       <c r="E27" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G27" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="H27" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="I27">
         <v>30</v>
@@ -3086,7 +2964,7 @@
         <v>28</v>
       </c>
       <c r="K27" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="L27" t="s">
         <v>29</v>
@@ -3098,7 +2976,7 @@
         <v>46</v>
       </c>
       <c r="O27" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -3106,22 +2984,22 @@
         <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C28" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D28" t="s">
         <v>57</v>
       </c>
       <c r="E28" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="G28" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="H28" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="I28">
         <v>12</v>
@@ -3130,7 +3008,7 @@
         <v>46</v>
       </c>
       <c r="K28" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="L28" t="s">
         <v>30</v>
@@ -3142,7 +3020,7 @@
         <v>46</v>
       </c>
       <c r="O28" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -3150,22 +3028,22 @@
         <v>16</v>
       </c>
       <c r="B29" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C29" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D29" t="s">
         <v>57</v>
       </c>
       <c r="E29" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="G29" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="H29" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="I29">
         <v>35</v>
@@ -3174,7 +3052,7 @@
         <v>32</v>
       </c>
       <c r="K29" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L29" t="s">
         <v>29</v>
@@ -3186,7 +3064,7 @@
         <v>46</v>
       </c>
       <c r="O29" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -3194,22 +3072,22 @@
         <v>16</v>
       </c>
       <c r="B30" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C30" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D30" t="s">
         <v>26</v>
       </c>
       <c r="E30" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G30" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="H30" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="I30">
         <v>35</v>
@@ -3218,7 +3096,7 @@
         <v>28</v>
       </c>
       <c r="K30" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L30" t="s">
         <v>29</v>
@@ -3230,7 +3108,7 @@
         <v>46</v>
       </c>
       <c r="O30" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -3238,22 +3116,22 @@
         <v>16</v>
       </c>
       <c r="B31" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C31" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D31" t="s">
         <v>47</v>
       </c>
       <c r="E31" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G31" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="H31" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="I31">
         <v>35</v>
@@ -3262,7 +3140,7 @@
         <v>30</v>
       </c>
       <c r="K31" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L31" t="s">
         <v>29</v>
@@ -3274,7 +3152,7 @@
         <v>46</v>
       </c>
       <c r="O31" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -3282,22 +3160,22 @@
         <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C32" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D32" t="s">
         <v>36</v>
       </c>
       <c r="E32" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="G32" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="H32" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="I32">
         <v>35</v>
@@ -3306,7 +3184,7 @@
         <v>35</v>
       </c>
       <c r="K32" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L32" t="s">
         <v>29</v>
@@ -3318,7 +3196,7 @@
         <v>46</v>
       </c>
       <c r="O32" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -3326,22 +3204,22 @@
         <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C33" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D33" t="s">
         <v>44</v>
       </c>
       <c r="E33" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="G33" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="H33" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="I33">
         <v>35</v>
@@ -3350,7 +3228,7 @@
         <v>30</v>
       </c>
       <c r="K33" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="L33" t="s">
         <v>29</v>
@@ -3362,7 +3240,7 @@
         <v>46</v>
       </c>
       <c r="O33" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -3385,268 +3263,268 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B2" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="C2" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D2" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="B3" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="C3" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D3" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="B4" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D4" t="s">
         <v>185</v>
-      </c>
-      <c r="D4" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="B5" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="C5" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D5" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="B6" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="C6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D6" t="s">
         <v>185</v>
-      </c>
-      <c r="D6" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="B7" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="C7" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D7" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B8" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="C8" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D8" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B9" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="C9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D9" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B10" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="C10" t="s">
+        <v>178</v>
+      </c>
+      <c r="D10" t="s">
         <v>185</v>
-      </c>
-      <c r="D10" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="B11" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="C11" t="s">
+        <v>178</v>
+      </c>
+      <c r="D11" t="s">
         <v>185</v>
-      </c>
-      <c r="D11" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B12" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="C12" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D12" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B13" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C13" t="s">
+        <v>178</v>
+      </c>
+      <c r="D13" t="s">
         <v>185</v>
-      </c>
-      <c r="D13" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B14" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="C14" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D14" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="B15" t="s">
+        <v>190</v>
+      </c>
+      <c r="C15" t="s">
+        <v>178</v>
+      </c>
+      <c r="D15" t="s">
         <v>197</v>
-      </c>
-      <c r="C15" t="s">
-        <v>185</v>
-      </c>
-      <c r="D15" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="B16" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="C16" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D16" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B17" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="C17" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D17" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="B18" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="C18" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D18" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="B19" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="C19" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D19" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -3669,19 +3547,19 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3692,13 +3570,13 @@
         <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>